<commit_message>
Updated OPEX & EBITDA page
</commit_message>
<xml_diff>
--- a/data/Сash_Flow_Actual.xlsx
+++ b/data/Сash_Flow_Actual.xlsx
@@ -4,10 +4,10 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22777" windowHeight="8590" tabRatio="924" activeTab="4"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22777" windowHeight="8665" tabRatio="924"/>
   </bookViews>
   <sheets>
-    <sheet name="Cash Flow Statment_Actual" sheetId="1" r:id="rId1"/>
+    <sheet name="Cash Flow Statement_Actual" sheetId="1" r:id="rId1"/>
     <sheet name="Sales_Actual" sheetId="2" r:id="rId2"/>
     <sheet name="COGS_Actual" sheetId="26" r:id="rId3"/>
     <sheet name="Working Capital_Actual" sheetId="34" r:id="rId4"/>

</xml_diff>

<commit_message>
Updated KPI & Monitoring Page
</commit_message>
<xml_diff>
--- a/data/Сash_Flow_Actual.xlsx
+++ b/data/Сash_Flow_Actual.xlsx
@@ -4,17 +4,18 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="2792" yWindow="0" windowWidth="23979" windowHeight="15151" tabRatio="924" activeTab="3"/>
+    <workbookView xWindow="2792" yWindow="0" windowWidth="23979" windowHeight="15151" tabRatio="924" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Cash Flow Statement_Actual" sheetId="1" r:id="rId1"/>
-    <sheet name="Sales_Actual" sheetId="2" r:id="rId2"/>
-    <sheet name="COGS_Actual" sheetId="26" r:id="rId3"/>
-    <sheet name="Working Capital_Actual" sheetId="34" r:id="rId4"/>
-    <sheet name="CapEx_Actual" sheetId="3" r:id="rId5"/>
-    <sheet name="Debt Schedule_Actual" sheetId="6" r:id="rId6"/>
-    <sheet name="DimDirection" sheetId="35" r:id="rId7"/>
-    <sheet name="OPEX_Actual" sheetId="36" r:id="rId8"/>
+    <sheet name="Balance Sheet_Actual" sheetId="37" r:id="rId2"/>
+    <sheet name="Sales_Actual" sheetId="2" r:id="rId3"/>
+    <sheet name="COGS_Actual" sheetId="26" r:id="rId4"/>
+    <sheet name="Working Capital_Actual" sheetId="34" r:id="rId5"/>
+    <sheet name="CapEx_Actual" sheetId="3" r:id="rId6"/>
+    <sheet name="Debt Schedule_Actual" sheetId="6" r:id="rId7"/>
+    <sheet name="DimDirection" sheetId="35" r:id="rId8"/>
+    <sheet name="OPEX_Actual" sheetId="36" r:id="rId9"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -29,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="97">
   <si>
     <t>Indicator</t>
   </si>
@@ -275,6 +276,51 @@
   </si>
   <si>
     <t>Cash Flow from Financing Activities</t>
+  </si>
+  <si>
+    <t>Cash and Cash Equivalents</t>
+  </si>
+  <si>
+    <t>Accounts Receivable</t>
+  </si>
+  <si>
+    <t>Inventory</t>
+  </si>
+  <si>
+    <t>Other Current Assets</t>
+  </si>
+  <si>
+    <t>Current Assets</t>
+  </si>
+  <si>
+    <t>Property Plant and Equipment</t>
+  </si>
+  <si>
+    <t>Other Non - current Assets</t>
+  </si>
+  <si>
+    <t>Total Assets</t>
+  </si>
+  <si>
+    <t>Short - term Debt</t>
+  </si>
+  <si>
+    <t>Long - term Debt</t>
+  </si>
+  <si>
+    <t>Accounts Payable</t>
+  </si>
+  <si>
+    <t>Other Current Liabilities</t>
+  </si>
+  <si>
+    <t>Current Liabilities</t>
+  </si>
+  <si>
+    <t>Total Liabilities</t>
+  </si>
+  <si>
+    <t>Total Equity</t>
   </si>
 </sst>
 </file>
@@ -721,7 +767,7 @@
     <xf numFmtId="167" fontId="13" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="167" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="95">
+  <cellXfs count="96">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -965,6 +1011,9 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="41"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="44">
     <cellStyle name="_macro (2)" xfId="3"/>
@@ -5397,6 +5446,2614 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:Z16"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="11.3" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="38.109375" style="13" customWidth="1"/>
+    <col min="2" max="2" width="12.44140625" style="13" customWidth="1"/>
+    <col min="3" max="3" width="11.44140625" style="13" customWidth="1"/>
+    <col min="4" max="4" width="13.109375" style="13" customWidth="1"/>
+    <col min="5" max="5" width="9.5546875" style="13" customWidth="1"/>
+    <col min="6" max="6" width="11.44140625" style="13" customWidth="1"/>
+    <col min="7" max="7" width="14" style="13" customWidth="1"/>
+    <col min="8" max="8" width="12" style="13" customWidth="1"/>
+    <col min="9" max="9" width="14.5546875" style="13" customWidth="1"/>
+    <col min="10" max="10" width="13" style="13" customWidth="1"/>
+    <col min="11" max="11" width="14" style="13" customWidth="1"/>
+    <col min="12" max="12" width="12" style="13" customWidth="1"/>
+    <col min="13" max="13" width="10" style="13" customWidth="1"/>
+    <col min="14" max="14" width="13" style="13" customWidth="1"/>
+    <col min="15" max="15" width="14" style="13" customWidth="1"/>
+    <col min="16" max="16" width="12" style="13" customWidth="1"/>
+    <col min="17" max="17" width="10" style="13" customWidth="1"/>
+    <col min="18" max="18" width="13" style="13" customWidth="1"/>
+    <col min="19" max="19" width="14" style="13" customWidth="1"/>
+    <col min="20" max="20" width="12" style="13" customWidth="1"/>
+    <col min="21" max="21" width="10" style="13" customWidth="1"/>
+    <col min="22" max="22" width="13" style="13" customWidth="1"/>
+    <col min="23" max="23" width="14" style="13" customWidth="1"/>
+    <col min="24" max="24" width="12" style="13" customWidth="1"/>
+    <col min="25" max="25" width="10" style="13" customWidth="1"/>
+    <col min="26" max="26" width="13" style="13" customWidth="1"/>
+    <col min="27" max="223" width="8.88671875" style="13"/>
+    <col min="224" max="224" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="225" max="225" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="226" max="226" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="227" max="227" width="10" style="13" customWidth="1"/>
+    <col min="228" max="228" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="229" max="229" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="230" max="230" width="13.44140625" style="13" customWidth="1"/>
+    <col min="231" max="231" width="12.109375" style="13" customWidth="1"/>
+    <col min="232" max="232" width="11.88671875" style="13" customWidth="1"/>
+    <col min="233" max="233" width="12.44140625" style="13" customWidth="1"/>
+    <col min="234" max="234" width="11.44140625" style="13" customWidth="1"/>
+    <col min="235" max="235" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="236" max="236" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="237" max="237" width="11.44140625" style="13" customWidth="1"/>
+    <col min="238" max="238" width="9.109375" style="13" customWidth="1"/>
+    <col min="239" max="240" width="10" style="13" customWidth="1"/>
+    <col min="241" max="241" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="242" max="479" width="8.88671875" style="13"/>
+    <col min="480" max="480" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="481" max="481" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="482" max="482" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="483" max="483" width="10" style="13" customWidth="1"/>
+    <col min="484" max="484" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="485" max="485" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="486" max="486" width="13.44140625" style="13" customWidth="1"/>
+    <col min="487" max="487" width="12.109375" style="13" customWidth="1"/>
+    <col min="488" max="488" width="11.88671875" style="13" customWidth="1"/>
+    <col min="489" max="489" width="12.44140625" style="13" customWidth="1"/>
+    <col min="490" max="490" width="11.44140625" style="13" customWidth="1"/>
+    <col min="491" max="491" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="492" max="492" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="493" max="493" width="11.44140625" style="13" customWidth="1"/>
+    <col min="494" max="494" width="9.109375" style="13" customWidth="1"/>
+    <col min="495" max="496" width="10" style="13" customWidth="1"/>
+    <col min="497" max="497" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="498" max="735" width="8.88671875" style="13"/>
+    <col min="736" max="736" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="737" max="737" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="738" max="738" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="739" max="739" width="10" style="13" customWidth="1"/>
+    <col min="740" max="740" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="741" max="741" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="742" max="742" width="13.44140625" style="13" customWidth="1"/>
+    <col min="743" max="743" width="12.109375" style="13" customWidth="1"/>
+    <col min="744" max="744" width="11.88671875" style="13" customWidth="1"/>
+    <col min="745" max="745" width="12.44140625" style="13" customWidth="1"/>
+    <col min="746" max="746" width="11.44140625" style="13" customWidth="1"/>
+    <col min="747" max="747" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="748" max="748" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="749" max="749" width="11.44140625" style="13" customWidth="1"/>
+    <col min="750" max="750" width="9.109375" style="13" customWidth="1"/>
+    <col min="751" max="752" width="10" style="13" customWidth="1"/>
+    <col min="753" max="753" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="754" max="991" width="8.88671875" style="13"/>
+    <col min="992" max="992" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="993" max="993" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="994" max="994" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="995" max="995" width="10" style="13" customWidth="1"/>
+    <col min="996" max="996" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="997" max="997" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="998" max="998" width="13.44140625" style="13" customWidth="1"/>
+    <col min="999" max="999" width="12.109375" style="13" customWidth="1"/>
+    <col min="1000" max="1000" width="11.88671875" style="13" customWidth="1"/>
+    <col min="1001" max="1001" width="12.44140625" style="13" customWidth="1"/>
+    <col min="1002" max="1002" width="11.44140625" style="13" customWidth="1"/>
+    <col min="1003" max="1003" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="1004" max="1004" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="1005" max="1005" width="11.44140625" style="13" customWidth="1"/>
+    <col min="1006" max="1006" width="9.109375" style="13" customWidth="1"/>
+    <col min="1007" max="1008" width="10" style="13" customWidth="1"/>
+    <col min="1009" max="1009" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="1010" max="1247" width="8.88671875" style="13"/>
+    <col min="1248" max="1248" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="1249" max="1249" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="1250" max="1250" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="1251" max="1251" width="10" style="13" customWidth="1"/>
+    <col min="1252" max="1252" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="1253" max="1253" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="1254" max="1254" width="13.44140625" style="13" customWidth="1"/>
+    <col min="1255" max="1255" width="12.109375" style="13" customWidth="1"/>
+    <col min="1256" max="1256" width="11.88671875" style="13" customWidth="1"/>
+    <col min="1257" max="1257" width="12.44140625" style="13" customWidth="1"/>
+    <col min="1258" max="1258" width="11.44140625" style="13" customWidth="1"/>
+    <col min="1259" max="1259" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="1260" max="1260" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="1261" max="1261" width="11.44140625" style="13" customWidth="1"/>
+    <col min="1262" max="1262" width="9.109375" style="13" customWidth="1"/>
+    <col min="1263" max="1264" width="10" style="13" customWidth="1"/>
+    <col min="1265" max="1265" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="1266" max="1503" width="8.88671875" style="13"/>
+    <col min="1504" max="1504" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="1505" max="1505" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="1506" max="1506" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="1507" max="1507" width="10" style="13" customWidth="1"/>
+    <col min="1508" max="1508" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="1509" max="1509" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="1510" max="1510" width="13.44140625" style="13" customWidth="1"/>
+    <col min="1511" max="1511" width="12.109375" style="13" customWidth="1"/>
+    <col min="1512" max="1512" width="11.88671875" style="13" customWidth="1"/>
+    <col min="1513" max="1513" width="12.44140625" style="13" customWidth="1"/>
+    <col min="1514" max="1514" width="11.44140625" style="13" customWidth="1"/>
+    <col min="1515" max="1515" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="1516" max="1516" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="1517" max="1517" width="11.44140625" style="13" customWidth="1"/>
+    <col min="1518" max="1518" width="9.109375" style="13" customWidth="1"/>
+    <col min="1519" max="1520" width="10" style="13" customWidth="1"/>
+    <col min="1521" max="1521" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="1522" max="1759" width="8.88671875" style="13"/>
+    <col min="1760" max="1760" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="1761" max="1761" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="1762" max="1762" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="1763" max="1763" width="10" style="13" customWidth="1"/>
+    <col min="1764" max="1764" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="1765" max="1765" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="1766" max="1766" width="13.44140625" style="13" customWidth="1"/>
+    <col min="1767" max="1767" width="12.109375" style="13" customWidth="1"/>
+    <col min="1768" max="1768" width="11.88671875" style="13" customWidth="1"/>
+    <col min="1769" max="1769" width="12.44140625" style="13" customWidth="1"/>
+    <col min="1770" max="1770" width="11.44140625" style="13" customWidth="1"/>
+    <col min="1771" max="1771" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="1772" max="1772" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="1773" max="1773" width="11.44140625" style="13" customWidth="1"/>
+    <col min="1774" max="1774" width="9.109375" style="13" customWidth="1"/>
+    <col min="1775" max="1776" width="10" style="13" customWidth="1"/>
+    <col min="1777" max="1777" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="1778" max="2015" width="8.88671875" style="13"/>
+    <col min="2016" max="2016" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="2017" max="2017" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="2018" max="2018" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="2019" max="2019" width="10" style="13" customWidth="1"/>
+    <col min="2020" max="2020" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="2021" max="2021" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="2022" max="2022" width="13.44140625" style="13" customWidth="1"/>
+    <col min="2023" max="2023" width="12.109375" style="13" customWidth="1"/>
+    <col min="2024" max="2024" width="11.88671875" style="13" customWidth="1"/>
+    <col min="2025" max="2025" width="12.44140625" style="13" customWidth="1"/>
+    <col min="2026" max="2026" width="11.44140625" style="13" customWidth="1"/>
+    <col min="2027" max="2027" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="2028" max="2028" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="2029" max="2029" width="11.44140625" style="13" customWidth="1"/>
+    <col min="2030" max="2030" width="9.109375" style="13" customWidth="1"/>
+    <col min="2031" max="2032" width="10" style="13" customWidth="1"/>
+    <col min="2033" max="2033" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="2034" max="2271" width="8.88671875" style="13"/>
+    <col min="2272" max="2272" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="2273" max="2273" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="2274" max="2274" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="2275" max="2275" width="10" style="13" customWidth="1"/>
+    <col min="2276" max="2276" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="2277" max="2277" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="2278" max="2278" width="13.44140625" style="13" customWidth="1"/>
+    <col min="2279" max="2279" width="12.109375" style="13" customWidth="1"/>
+    <col min="2280" max="2280" width="11.88671875" style="13" customWidth="1"/>
+    <col min="2281" max="2281" width="12.44140625" style="13" customWidth="1"/>
+    <col min="2282" max="2282" width="11.44140625" style="13" customWidth="1"/>
+    <col min="2283" max="2283" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="2284" max="2284" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="2285" max="2285" width="11.44140625" style="13" customWidth="1"/>
+    <col min="2286" max="2286" width="9.109375" style="13" customWidth="1"/>
+    <col min="2287" max="2288" width="10" style="13" customWidth="1"/>
+    <col min="2289" max="2289" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="2290" max="2527" width="8.88671875" style="13"/>
+    <col min="2528" max="2528" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="2529" max="2529" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="2530" max="2530" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="2531" max="2531" width="10" style="13" customWidth="1"/>
+    <col min="2532" max="2532" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="2533" max="2533" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="2534" max="2534" width="13.44140625" style="13" customWidth="1"/>
+    <col min="2535" max="2535" width="12.109375" style="13" customWidth="1"/>
+    <col min="2536" max="2536" width="11.88671875" style="13" customWidth="1"/>
+    <col min="2537" max="2537" width="12.44140625" style="13" customWidth="1"/>
+    <col min="2538" max="2538" width="11.44140625" style="13" customWidth="1"/>
+    <col min="2539" max="2539" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="2540" max="2540" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="2541" max="2541" width="11.44140625" style="13" customWidth="1"/>
+    <col min="2542" max="2542" width="9.109375" style="13" customWidth="1"/>
+    <col min="2543" max="2544" width="10" style="13" customWidth="1"/>
+    <col min="2545" max="2545" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="2546" max="2783" width="8.88671875" style="13"/>
+    <col min="2784" max="2784" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="2785" max="2785" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="2786" max="2786" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="2787" max="2787" width="10" style="13" customWidth="1"/>
+    <col min="2788" max="2788" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="2789" max="2789" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="2790" max="2790" width="13.44140625" style="13" customWidth="1"/>
+    <col min="2791" max="2791" width="12.109375" style="13" customWidth="1"/>
+    <col min="2792" max="2792" width="11.88671875" style="13" customWidth="1"/>
+    <col min="2793" max="2793" width="12.44140625" style="13" customWidth="1"/>
+    <col min="2794" max="2794" width="11.44140625" style="13" customWidth="1"/>
+    <col min="2795" max="2795" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="2796" max="2796" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="2797" max="2797" width="11.44140625" style="13" customWidth="1"/>
+    <col min="2798" max="2798" width="9.109375" style="13" customWidth="1"/>
+    <col min="2799" max="2800" width="10" style="13" customWidth="1"/>
+    <col min="2801" max="2801" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="2802" max="3039" width="8.88671875" style="13"/>
+    <col min="3040" max="3040" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="3041" max="3041" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="3042" max="3042" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="3043" max="3043" width="10" style="13" customWidth="1"/>
+    <col min="3044" max="3044" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="3045" max="3045" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="3046" max="3046" width="13.44140625" style="13" customWidth="1"/>
+    <col min="3047" max="3047" width="12.109375" style="13" customWidth="1"/>
+    <col min="3048" max="3048" width="11.88671875" style="13" customWidth="1"/>
+    <col min="3049" max="3049" width="12.44140625" style="13" customWidth="1"/>
+    <col min="3050" max="3050" width="11.44140625" style="13" customWidth="1"/>
+    <col min="3051" max="3051" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="3052" max="3052" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="3053" max="3053" width="11.44140625" style="13" customWidth="1"/>
+    <col min="3054" max="3054" width="9.109375" style="13" customWidth="1"/>
+    <col min="3055" max="3056" width="10" style="13" customWidth="1"/>
+    <col min="3057" max="3057" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="3058" max="3295" width="8.88671875" style="13"/>
+    <col min="3296" max="3296" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="3297" max="3297" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="3298" max="3298" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="3299" max="3299" width="10" style="13" customWidth="1"/>
+    <col min="3300" max="3300" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="3301" max="3301" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="3302" max="3302" width="13.44140625" style="13" customWidth="1"/>
+    <col min="3303" max="3303" width="12.109375" style="13" customWidth="1"/>
+    <col min="3304" max="3304" width="11.88671875" style="13" customWidth="1"/>
+    <col min="3305" max="3305" width="12.44140625" style="13" customWidth="1"/>
+    <col min="3306" max="3306" width="11.44140625" style="13" customWidth="1"/>
+    <col min="3307" max="3307" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="3308" max="3308" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="3309" max="3309" width="11.44140625" style="13" customWidth="1"/>
+    <col min="3310" max="3310" width="9.109375" style="13" customWidth="1"/>
+    <col min="3311" max="3312" width="10" style="13" customWidth="1"/>
+    <col min="3313" max="3313" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="3314" max="3551" width="8.88671875" style="13"/>
+    <col min="3552" max="3552" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="3553" max="3553" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="3554" max="3554" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="3555" max="3555" width="10" style="13" customWidth="1"/>
+    <col min="3556" max="3556" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="3557" max="3557" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="3558" max="3558" width="13.44140625" style="13" customWidth="1"/>
+    <col min="3559" max="3559" width="12.109375" style="13" customWidth="1"/>
+    <col min="3560" max="3560" width="11.88671875" style="13" customWidth="1"/>
+    <col min="3561" max="3561" width="12.44140625" style="13" customWidth="1"/>
+    <col min="3562" max="3562" width="11.44140625" style="13" customWidth="1"/>
+    <col min="3563" max="3563" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="3564" max="3564" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="3565" max="3565" width="11.44140625" style="13" customWidth="1"/>
+    <col min="3566" max="3566" width="9.109375" style="13" customWidth="1"/>
+    <col min="3567" max="3568" width="10" style="13" customWidth="1"/>
+    <col min="3569" max="3569" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="3570" max="3807" width="8.88671875" style="13"/>
+    <col min="3808" max="3808" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="3809" max="3809" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="3810" max="3810" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="3811" max="3811" width="10" style="13" customWidth="1"/>
+    <col min="3812" max="3812" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="3813" max="3813" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="3814" max="3814" width="13.44140625" style="13" customWidth="1"/>
+    <col min="3815" max="3815" width="12.109375" style="13" customWidth="1"/>
+    <col min="3816" max="3816" width="11.88671875" style="13" customWidth="1"/>
+    <col min="3817" max="3817" width="12.44140625" style="13" customWidth="1"/>
+    <col min="3818" max="3818" width="11.44140625" style="13" customWidth="1"/>
+    <col min="3819" max="3819" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="3820" max="3820" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="3821" max="3821" width="11.44140625" style="13" customWidth="1"/>
+    <col min="3822" max="3822" width="9.109375" style="13" customWidth="1"/>
+    <col min="3823" max="3824" width="10" style="13" customWidth="1"/>
+    <col min="3825" max="3825" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="3826" max="4063" width="8.88671875" style="13"/>
+    <col min="4064" max="4064" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="4065" max="4065" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="4066" max="4066" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="4067" max="4067" width="10" style="13" customWidth="1"/>
+    <col min="4068" max="4068" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="4069" max="4069" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="4070" max="4070" width="13.44140625" style="13" customWidth="1"/>
+    <col min="4071" max="4071" width="12.109375" style="13" customWidth="1"/>
+    <col min="4072" max="4072" width="11.88671875" style="13" customWidth="1"/>
+    <col min="4073" max="4073" width="12.44140625" style="13" customWidth="1"/>
+    <col min="4074" max="4074" width="11.44140625" style="13" customWidth="1"/>
+    <col min="4075" max="4075" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="4076" max="4076" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="4077" max="4077" width="11.44140625" style="13" customWidth="1"/>
+    <col min="4078" max="4078" width="9.109375" style="13" customWidth="1"/>
+    <col min="4079" max="4080" width="10" style="13" customWidth="1"/>
+    <col min="4081" max="4081" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="4082" max="4319" width="8.88671875" style="13"/>
+    <col min="4320" max="4320" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="4321" max="4321" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="4322" max="4322" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="4323" max="4323" width="10" style="13" customWidth="1"/>
+    <col min="4324" max="4324" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="4325" max="4325" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="4326" max="4326" width="13.44140625" style="13" customWidth="1"/>
+    <col min="4327" max="4327" width="12.109375" style="13" customWidth="1"/>
+    <col min="4328" max="4328" width="11.88671875" style="13" customWidth="1"/>
+    <col min="4329" max="4329" width="12.44140625" style="13" customWidth="1"/>
+    <col min="4330" max="4330" width="11.44140625" style="13" customWidth="1"/>
+    <col min="4331" max="4331" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="4332" max="4332" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="4333" max="4333" width="11.44140625" style="13" customWidth="1"/>
+    <col min="4334" max="4334" width="9.109375" style="13" customWidth="1"/>
+    <col min="4335" max="4336" width="10" style="13" customWidth="1"/>
+    <col min="4337" max="4337" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="4338" max="4575" width="8.88671875" style="13"/>
+    <col min="4576" max="4576" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="4577" max="4577" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="4578" max="4578" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="4579" max="4579" width="10" style="13" customWidth="1"/>
+    <col min="4580" max="4580" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="4581" max="4581" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="4582" max="4582" width="13.44140625" style="13" customWidth="1"/>
+    <col min="4583" max="4583" width="12.109375" style="13" customWidth="1"/>
+    <col min="4584" max="4584" width="11.88671875" style="13" customWidth="1"/>
+    <col min="4585" max="4585" width="12.44140625" style="13" customWidth="1"/>
+    <col min="4586" max="4586" width="11.44140625" style="13" customWidth="1"/>
+    <col min="4587" max="4587" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="4588" max="4588" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="4589" max="4589" width="11.44140625" style="13" customWidth="1"/>
+    <col min="4590" max="4590" width="9.109375" style="13" customWidth="1"/>
+    <col min="4591" max="4592" width="10" style="13" customWidth="1"/>
+    <col min="4593" max="4593" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="4594" max="4831" width="8.88671875" style="13"/>
+    <col min="4832" max="4832" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="4833" max="4833" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="4834" max="4834" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="4835" max="4835" width="10" style="13" customWidth="1"/>
+    <col min="4836" max="4836" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="4837" max="4837" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="4838" max="4838" width="13.44140625" style="13" customWidth="1"/>
+    <col min="4839" max="4839" width="12.109375" style="13" customWidth="1"/>
+    <col min="4840" max="4840" width="11.88671875" style="13" customWidth="1"/>
+    <col min="4841" max="4841" width="12.44140625" style="13" customWidth="1"/>
+    <col min="4842" max="4842" width="11.44140625" style="13" customWidth="1"/>
+    <col min="4843" max="4843" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="4844" max="4844" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="4845" max="4845" width="11.44140625" style="13" customWidth="1"/>
+    <col min="4846" max="4846" width="9.109375" style="13" customWidth="1"/>
+    <col min="4847" max="4848" width="10" style="13" customWidth="1"/>
+    <col min="4849" max="4849" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="4850" max="5087" width="8.88671875" style="13"/>
+    <col min="5088" max="5088" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="5089" max="5089" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="5090" max="5090" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="5091" max="5091" width="10" style="13" customWidth="1"/>
+    <col min="5092" max="5092" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="5093" max="5093" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="5094" max="5094" width="13.44140625" style="13" customWidth="1"/>
+    <col min="5095" max="5095" width="12.109375" style="13" customWidth="1"/>
+    <col min="5096" max="5096" width="11.88671875" style="13" customWidth="1"/>
+    <col min="5097" max="5097" width="12.44140625" style="13" customWidth="1"/>
+    <col min="5098" max="5098" width="11.44140625" style="13" customWidth="1"/>
+    <col min="5099" max="5099" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="5100" max="5100" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="5101" max="5101" width="11.44140625" style="13" customWidth="1"/>
+    <col min="5102" max="5102" width="9.109375" style="13" customWidth="1"/>
+    <col min="5103" max="5104" width="10" style="13" customWidth="1"/>
+    <col min="5105" max="5105" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="5106" max="5343" width="8.88671875" style="13"/>
+    <col min="5344" max="5344" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="5345" max="5345" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="5346" max="5346" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="5347" max="5347" width="10" style="13" customWidth="1"/>
+    <col min="5348" max="5348" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="5349" max="5349" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="5350" max="5350" width="13.44140625" style="13" customWidth="1"/>
+    <col min="5351" max="5351" width="12.109375" style="13" customWidth="1"/>
+    <col min="5352" max="5352" width="11.88671875" style="13" customWidth="1"/>
+    <col min="5353" max="5353" width="12.44140625" style="13" customWidth="1"/>
+    <col min="5354" max="5354" width="11.44140625" style="13" customWidth="1"/>
+    <col min="5355" max="5355" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="5356" max="5356" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="5357" max="5357" width="11.44140625" style="13" customWidth="1"/>
+    <col min="5358" max="5358" width="9.109375" style="13" customWidth="1"/>
+    <col min="5359" max="5360" width="10" style="13" customWidth="1"/>
+    <col min="5361" max="5361" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="5362" max="5599" width="8.88671875" style="13"/>
+    <col min="5600" max="5600" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="5601" max="5601" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="5602" max="5602" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="5603" max="5603" width="10" style="13" customWidth="1"/>
+    <col min="5604" max="5604" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="5605" max="5605" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="5606" max="5606" width="13.44140625" style="13" customWidth="1"/>
+    <col min="5607" max="5607" width="12.109375" style="13" customWidth="1"/>
+    <col min="5608" max="5608" width="11.88671875" style="13" customWidth="1"/>
+    <col min="5609" max="5609" width="12.44140625" style="13" customWidth="1"/>
+    <col min="5610" max="5610" width="11.44140625" style="13" customWidth="1"/>
+    <col min="5611" max="5611" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="5612" max="5612" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="5613" max="5613" width="11.44140625" style="13" customWidth="1"/>
+    <col min="5614" max="5614" width="9.109375" style="13" customWidth="1"/>
+    <col min="5615" max="5616" width="10" style="13" customWidth="1"/>
+    <col min="5617" max="5617" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="5618" max="5855" width="8.88671875" style="13"/>
+    <col min="5856" max="5856" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="5857" max="5857" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="5858" max="5858" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="5859" max="5859" width="10" style="13" customWidth="1"/>
+    <col min="5860" max="5860" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="5861" max="5861" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="5862" max="5862" width="13.44140625" style="13" customWidth="1"/>
+    <col min="5863" max="5863" width="12.109375" style="13" customWidth="1"/>
+    <col min="5864" max="5864" width="11.88671875" style="13" customWidth="1"/>
+    <col min="5865" max="5865" width="12.44140625" style="13" customWidth="1"/>
+    <col min="5866" max="5866" width="11.44140625" style="13" customWidth="1"/>
+    <col min="5867" max="5867" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="5868" max="5868" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="5869" max="5869" width="11.44140625" style="13" customWidth="1"/>
+    <col min="5870" max="5870" width="9.109375" style="13" customWidth="1"/>
+    <col min="5871" max="5872" width="10" style="13" customWidth="1"/>
+    <col min="5873" max="5873" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="5874" max="6111" width="8.88671875" style="13"/>
+    <col min="6112" max="6112" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="6113" max="6113" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="6114" max="6114" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="6115" max="6115" width="10" style="13" customWidth="1"/>
+    <col min="6116" max="6116" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="6117" max="6117" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="6118" max="6118" width="13.44140625" style="13" customWidth="1"/>
+    <col min="6119" max="6119" width="12.109375" style="13" customWidth="1"/>
+    <col min="6120" max="6120" width="11.88671875" style="13" customWidth="1"/>
+    <col min="6121" max="6121" width="12.44140625" style="13" customWidth="1"/>
+    <col min="6122" max="6122" width="11.44140625" style="13" customWidth="1"/>
+    <col min="6123" max="6123" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="6124" max="6124" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="6125" max="6125" width="11.44140625" style="13" customWidth="1"/>
+    <col min="6126" max="6126" width="9.109375" style="13" customWidth="1"/>
+    <col min="6127" max="6128" width="10" style="13" customWidth="1"/>
+    <col min="6129" max="6129" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="6130" max="6367" width="8.88671875" style="13"/>
+    <col min="6368" max="6368" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="6369" max="6369" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="6370" max="6370" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="6371" max="6371" width="10" style="13" customWidth="1"/>
+    <col min="6372" max="6372" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="6373" max="6373" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="6374" max="6374" width="13.44140625" style="13" customWidth="1"/>
+    <col min="6375" max="6375" width="12.109375" style="13" customWidth="1"/>
+    <col min="6376" max="6376" width="11.88671875" style="13" customWidth="1"/>
+    <col min="6377" max="6377" width="12.44140625" style="13" customWidth="1"/>
+    <col min="6378" max="6378" width="11.44140625" style="13" customWidth="1"/>
+    <col min="6379" max="6379" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="6380" max="6380" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="6381" max="6381" width="11.44140625" style="13" customWidth="1"/>
+    <col min="6382" max="6382" width="9.109375" style="13" customWidth="1"/>
+    <col min="6383" max="6384" width="10" style="13" customWidth="1"/>
+    <col min="6385" max="6385" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="6386" max="6623" width="8.88671875" style="13"/>
+    <col min="6624" max="6624" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="6625" max="6625" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="6626" max="6626" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="6627" max="6627" width="10" style="13" customWidth="1"/>
+    <col min="6628" max="6628" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="6629" max="6629" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="6630" max="6630" width="13.44140625" style="13" customWidth="1"/>
+    <col min="6631" max="6631" width="12.109375" style="13" customWidth="1"/>
+    <col min="6632" max="6632" width="11.88671875" style="13" customWidth="1"/>
+    <col min="6633" max="6633" width="12.44140625" style="13" customWidth="1"/>
+    <col min="6634" max="6634" width="11.44140625" style="13" customWidth="1"/>
+    <col min="6635" max="6635" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="6636" max="6636" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="6637" max="6637" width="11.44140625" style="13" customWidth="1"/>
+    <col min="6638" max="6638" width="9.109375" style="13" customWidth="1"/>
+    <col min="6639" max="6640" width="10" style="13" customWidth="1"/>
+    <col min="6641" max="6641" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="6642" max="6879" width="8.88671875" style="13"/>
+    <col min="6880" max="6880" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="6881" max="6881" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="6882" max="6882" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="6883" max="6883" width="10" style="13" customWidth="1"/>
+    <col min="6884" max="6884" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="6885" max="6885" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="6886" max="6886" width="13.44140625" style="13" customWidth="1"/>
+    <col min="6887" max="6887" width="12.109375" style="13" customWidth="1"/>
+    <col min="6888" max="6888" width="11.88671875" style="13" customWidth="1"/>
+    <col min="6889" max="6889" width="12.44140625" style="13" customWidth="1"/>
+    <col min="6890" max="6890" width="11.44140625" style="13" customWidth="1"/>
+    <col min="6891" max="6891" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="6892" max="6892" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="6893" max="6893" width="11.44140625" style="13" customWidth="1"/>
+    <col min="6894" max="6894" width="9.109375" style="13" customWidth="1"/>
+    <col min="6895" max="6896" width="10" style="13" customWidth="1"/>
+    <col min="6897" max="6897" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="6898" max="7135" width="8.88671875" style="13"/>
+    <col min="7136" max="7136" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="7137" max="7137" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="7138" max="7138" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="7139" max="7139" width="10" style="13" customWidth="1"/>
+    <col min="7140" max="7140" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="7141" max="7141" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="7142" max="7142" width="13.44140625" style="13" customWidth="1"/>
+    <col min="7143" max="7143" width="12.109375" style="13" customWidth="1"/>
+    <col min="7144" max="7144" width="11.88671875" style="13" customWidth="1"/>
+    <col min="7145" max="7145" width="12.44140625" style="13" customWidth="1"/>
+    <col min="7146" max="7146" width="11.44140625" style="13" customWidth="1"/>
+    <col min="7147" max="7147" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="7148" max="7148" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="7149" max="7149" width="11.44140625" style="13" customWidth="1"/>
+    <col min="7150" max="7150" width="9.109375" style="13" customWidth="1"/>
+    <col min="7151" max="7152" width="10" style="13" customWidth="1"/>
+    <col min="7153" max="7153" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="7154" max="7391" width="8.88671875" style="13"/>
+    <col min="7392" max="7392" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="7393" max="7393" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="7394" max="7394" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="7395" max="7395" width="10" style="13" customWidth="1"/>
+    <col min="7396" max="7396" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="7397" max="7397" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="7398" max="7398" width="13.44140625" style="13" customWidth="1"/>
+    <col min="7399" max="7399" width="12.109375" style="13" customWidth="1"/>
+    <col min="7400" max="7400" width="11.88671875" style="13" customWidth="1"/>
+    <col min="7401" max="7401" width="12.44140625" style="13" customWidth="1"/>
+    <col min="7402" max="7402" width="11.44140625" style="13" customWidth="1"/>
+    <col min="7403" max="7403" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="7404" max="7404" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="7405" max="7405" width="11.44140625" style="13" customWidth="1"/>
+    <col min="7406" max="7406" width="9.109375" style="13" customWidth="1"/>
+    <col min="7407" max="7408" width="10" style="13" customWidth="1"/>
+    <col min="7409" max="7409" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="7410" max="7647" width="8.88671875" style="13"/>
+    <col min="7648" max="7648" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="7649" max="7649" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="7650" max="7650" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="7651" max="7651" width="10" style="13" customWidth="1"/>
+    <col min="7652" max="7652" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="7653" max="7653" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="7654" max="7654" width="13.44140625" style="13" customWidth="1"/>
+    <col min="7655" max="7655" width="12.109375" style="13" customWidth="1"/>
+    <col min="7656" max="7656" width="11.88671875" style="13" customWidth="1"/>
+    <col min="7657" max="7657" width="12.44140625" style="13" customWidth="1"/>
+    <col min="7658" max="7658" width="11.44140625" style="13" customWidth="1"/>
+    <col min="7659" max="7659" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="7660" max="7660" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="7661" max="7661" width="11.44140625" style="13" customWidth="1"/>
+    <col min="7662" max="7662" width="9.109375" style="13" customWidth="1"/>
+    <col min="7663" max="7664" width="10" style="13" customWidth="1"/>
+    <col min="7665" max="7665" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="7666" max="7903" width="8.88671875" style="13"/>
+    <col min="7904" max="7904" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="7905" max="7905" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="7906" max="7906" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="7907" max="7907" width="10" style="13" customWidth="1"/>
+    <col min="7908" max="7908" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="7909" max="7909" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="7910" max="7910" width="13.44140625" style="13" customWidth="1"/>
+    <col min="7911" max="7911" width="12.109375" style="13" customWidth="1"/>
+    <col min="7912" max="7912" width="11.88671875" style="13" customWidth="1"/>
+    <col min="7913" max="7913" width="12.44140625" style="13" customWidth="1"/>
+    <col min="7914" max="7914" width="11.44140625" style="13" customWidth="1"/>
+    <col min="7915" max="7915" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="7916" max="7916" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="7917" max="7917" width="11.44140625" style="13" customWidth="1"/>
+    <col min="7918" max="7918" width="9.109375" style="13" customWidth="1"/>
+    <col min="7919" max="7920" width="10" style="13" customWidth="1"/>
+    <col min="7921" max="7921" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="7922" max="8159" width="8.88671875" style="13"/>
+    <col min="8160" max="8160" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="8161" max="8161" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="8162" max="8162" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="8163" max="8163" width="10" style="13" customWidth="1"/>
+    <col min="8164" max="8164" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="8165" max="8165" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="8166" max="8166" width="13.44140625" style="13" customWidth="1"/>
+    <col min="8167" max="8167" width="12.109375" style="13" customWidth="1"/>
+    <col min="8168" max="8168" width="11.88671875" style="13" customWidth="1"/>
+    <col min="8169" max="8169" width="12.44140625" style="13" customWidth="1"/>
+    <col min="8170" max="8170" width="11.44140625" style="13" customWidth="1"/>
+    <col min="8171" max="8171" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="8172" max="8172" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="8173" max="8173" width="11.44140625" style="13" customWidth="1"/>
+    <col min="8174" max="8174" width="9.109375" style="13" customWidth="1"/>
+    <col min="8175" max="8176" width="10" style="13" customWidth="1"/>
+    <col min="8177" max="8177" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="8178" max="8415" width="8.88671875" style="13"/>
+    <col min="8416" max="8416" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="8417" max="8417" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="8418" max="8418" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="8419" max="8419" width="10" style="13" customWidth="1"/>
+    <col min="8420" max="8420" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="8421" max="8421" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="8422" max="8422" width="13.44140625" style="13" customWidth="1"/>
+    <col min="8423" max="8423" width="12.109375" style="13" customWidth="1"/>
+    <col min="8424" max="8424" width="11.88671875" style="13" customWidth="1"/>
+    <col min="8425" max="8425" width="12.44140625" style="13" customWidth="1"/>
+    <col min="8426" max="8426" width="11.44140625" style="13" customWidth="1"/>
+    <col min="8427" max="8427" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="8428" max="8428" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="8429" max="8429" width="11.44140625" style="13" customWidth="1"/>
+    <col min="8430" max="8430" width="9.109375" style="13" customWidth="1"/>
+    <col min="8431" max="8432" width="10" style="13" customWidth="1"/>
+    <col min="8433" max="8433" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="8434" max="8671" width="8.88671875" style="13"/>
+    <col min="8672" max="8672" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="8673" max="8673" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="8674" max="8674" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="8675" max="8675" width="10" style="13" customWidth="1"/>
+    <col min="8676" max="8676" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="8677" max="8677" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="8678" max="8678" width="13.44140625" style="13" customWidth="1"/>
+    <col min="8679" max="8679" width="12.109375" style="13" customWidth="1"/>
+    <col min="8680" max="8680" width="11.88671875" style="13" customWidth="1"/>
+    <col min="8681" max="8681" width="12.44140625" style="13" customWidth="1"/>
+    <col min="8682" max="8682" width="11.44140625" style="13" customWidth="1"/>
+    <col min="8683" max="8683" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="8684" max="8684" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="8685" max="8685" width="11.44140625" style="13" customWidth="1"/>
+    <col min="8686" max="8686" width="9.109375" style="13" customWidth="1"/>
+    <col min="8687" max="8688" width="10" style="13" customWidth="1"/>
+    <col min="8689" max="8689" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="8690" max="8927" width="8.88671875" style="13"/>
+    <col min="8928" max="8928" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="8929" max="8929" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="8930" max="8930" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="8931" max="8931" width="10" style="13" customWidth="1"/>
+    <col min="8932" max="8932" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="8933" max="8933" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="8934" max="8934" width="13.44140625" style="13" customWidth="1"/>
+    <col min="8935" max="8935" width="12.109375" style="13" customWidth="1"/>
+    <col min="8936" max="8936" width="11.88671875" style="13" customWidth="1"/>
+    <col min="8937" max="8937" width="12.44140625" style="13" customWidth="1"/>
+    <col min="8938" max="8938" width="11.44140625" style="13" customWidth="1"/>
+    <col min="8939" max="8939" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="8940" max="8940" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="8941" max="8941" width="11.44140625" style="13" customWidth="1"/>
+    <col min="8942" max="8942" width="9.109375" style="13" customWidth="1"/>
+    <col min="8943" max="8944" width="10" style="13" customWidth="1"/>
+    <col min="8945" max="8945" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="8946" max="9183" width="8.88671875" style="13"/>
+    <col min="9184" max="9184" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="9185" max="9185" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="9186" max="9186" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="9187" max="9187" width="10" style="13" customWidth="1"/>
+    <col min="9188" max="9188" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="9189" max="9189" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="9190" max="9190" width="13.44140625" style="13" customWidth="1"/>
+    <col min="9191" max="9191" width="12.109375" style="13" customWidth="1"/>
+    <col min="9192" max="9192" width="11.88671875" style="13" customWidth="1"/>
+    <col min="9193" max="9193" width="12.44140625" style="13" customWidth="1"/>
+    <col min="9194" max="9194" width="11.44140625" style="13" customWidth="1"/>
+    <col min="9195" max="9195" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="9196" max="9196" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="9197" max="9197" width="11.44140625" style="13" customWidth="1"/>
+    <col min="9198" max="9198" width="9.109375" style="13" customWidth="1"/>
+    <col min="9199" max="9200" width="10" style="13" customWidth="1"/>
+    <col min="9201" max="9201" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="9202" max="9439" width="8.88671875" style="13"/>
+    <col min="9440" max="9440" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="9441" max="9441" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="9442" max="9442" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="9443" max="9443" width="10" style="13" customWidth="1"/>
+    <col min="9444" max="9444" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="9445" max="9445" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="9446" max="9446" width="13.44140625" style="13" customWidth="1"/>
+    <col min="9447" max="9447" width="12.109375" style="13" customWidth="1"/>
+    <col min="9448" max="9448" width="11.88671875" style="13" customWidth="1"/>
+    <col min="9449" max="9449" width="12.44140625" style="13" customWidth="1"/>
+    <col min="9450" max="9450" width="11.44140625" style="13" customWidth="1"/>
+    <col min="9451" max="9451" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="9452" max="9452" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="9453" max="9453" width="11.44140625" style="13" customWidth="1"/>
+    <col min="9454" max="9454" width="9.109375" style="13" customWidth="1"/>
+    <col min="9455" max="9456" width="10" style="13" customWidth="1"/>
+    <col min="9457" max="9457" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="9458" max="9695" width="8.88671875" style="13"/>
+    <col min="9696" max="9696" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="9697" max="9697" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="9698" max="9698" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="9699" max="9699" width="10" style="13" customWidth="1"/>
+    <col min="9700" max="9700" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="9701" max="9701" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="9702" max="9702" width="13.44140625" style="13" customWidth="1"/>
+    <col min="9703" max="9703" width="12.109375" style="13" customWidth="1"/>
+    <col min="9704" max="9704" width="11.88671875" style="13" customWidth="1"/>
+    <col min="9705" max="9705" width="12.44140625" style="13" customWidth="1"/>
+    <col min="9706" max="9706" width="11.44140625" style="13" customWidth="1"/>
+    <col min="9707" max="9707" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="9708" max="9708" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="9709" max="9709" width="11.44140625" style="13" customWidth="1"/>
+    <col min="9710" max="9710" width="9.109375" style="13" customWidth="1"/>
+    <col min="9711" max="9712" width="10" style="13" customWidth="1"/>
+    <col min="9713" max="9713" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="9714" max="9951" width="8.88671875" style="13"/>
+    <col min="9952" max="9952" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="9953" max="9953" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="9954" max="9954" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="9955" max="9955" width="10" style="13" customWidth="1"/>
+    <col min="9956" max="9956" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="9957" max="9957" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="9958" max="9958" width="13.44140625" style="13" customWidth="1"/>
+    <col min="9959" max="9959" width="12.109375" style="13" customWidth="1"/>
+    <col min="9960" max="9960" width="11.88671875" style="13" customWidth="1"/>
+    <col min="9961" max="9961" width="12.44140625" style="13" customWidth="1"/>
+    <col min="9962" max="9962" width="11.44140625" style="13" customWidth="1"/>
+    <col min="9963" max="9963" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="9964" max="9964" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="9965" max="9965" width="11.44140625" style="13" customWidth="1"/>
+    <col min="9966" max="9966" width="9.109375" style="13" customWidth="1"/>
+    <col min="9967" max="9968" width="10" style="13" customWidth="1"/>
+    <col min="9969" max="9969" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="9970" max="10207" width="8.88671875" style="13"/>
+    <col min="10208" max="10208" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="10209" max="10209" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="10210" max="10210" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="10211" max="10211" width="10" style="13" customWidth="1"/>
+    <col min="10212" max="10212" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="10213" max="10213" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="10214" max="10214" width="13.44140625" style="13" customWidth="1"/>
+    <col min="10215" max="10215" width="12.109375" style="13" customWidth="1"/>
+    <col min="10216" max="10216" width="11.88671875" style="13" customWidth="1"/>
+    <col min="10217" max="10217" width="12.44140625" style="13" customWidth="1"/>
+    <col min="10218" max="10218" width="11.44140625" style="13" customWidth="1"/>
+    <col min="10219" max="10219" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="10220" max="10220" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="10221" max="10221" width="11.44140625" style="13" customWidth="1"/>
+    <col min="10222" max="10222" width="9.109375" style="13" customWidth="1"/>
+    <col min="10223" max="10224" width="10" style="13" customWidth="1"/>
+    <col min="10225" max="10225" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="10226" max="10463" width="8.88671875" style="13"/>
+    <col min="10464" max="10464" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="10465" max="10465" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="10466" max="10466" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="10467" max="10467" width="10" style="13" customWidth="1"/>
+    <col min="10468" max="10468" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="10469" max="10469" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="10470" max="10470" width="13.44140625" style="13" customWidth="1"/>
+    <col min="10471" max="10471" width="12.109375" style="13" customWidth="1"/>
+    <col min="10472" max="10472" width="11.88671875" style="13" customWidth="1"/>
+    <col min="10473" max="10473" width="12.44140625" style="13" customWidth="1"/>
+    <col min="10474" max="10474" width="11.44140625" style="13" customWidth="1"/>
+    <col min="10475" max="10475" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="10476" max="10476" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="10477" max="10477" width="11.44140625" style="13" customWidth="1"/>
+    <col min="10478" max="10478" width="9.109375" style="13" customWidth="1"/>
+    <col min="10479" max="10480" width="10" style="13" customWidth="1"/>
+    <col min="10481" max="10481" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="10482" max="10719" width="8.88671875" style="13"/>
+    <col min="10720" max="10720" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="10721" max="10721" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="10722" max="10722" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="10723" max="10723" width="10" style="13" customWidth="1"/>
+    <col min="10724" max="10724" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="10725" max="10725" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="10726" max="10726" width="13.44140625" style="13" customWidth="1"/>
+    <col min="10727" max="10727" width="12.109375" style="13" customWidth="1"/>
+    <col min="10728" max="10728" width="11.88671875" style="13" customWidth="1"/>
+    <col min="10729" max="10729" width="12.44140625" style="13" customWidth="1"/>
+    <col min="10730" max="10730" width="11.44140625" style="13" customWidth="1"/>
+    <col min="10731" max="10731" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="10732" max="10732" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="10733" max="10733" width="11.44140625" style="13" customWidth="1"/>
+    <col min="10734" max="10734" width="9.109375" style="13" customWidth="1"/>
+    <col min="10735" max="10736" width="10" style="13" customWidth="1"/>
+    <col min="10737" max="10737" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="10738" max="10975" width="8.88671875" style="13"/>
+    <col min="10976" max="10976" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="10977" max="10977" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="10978" max="10978" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="10979" max="10979" width="10" style="13" customWidth="1"/>
+    <col min="10980" max="10980" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="10981" max="10981" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="10982" max="10982" width="13.44140625" style="13" customWidth="1"/>
+    <col min="10983" max="10983" width="12.109375" style="13" customWidth="1"/>
+    <col min="10984" max="10984" width="11.88671875" style="13" customWidth="1"/>
+    <col min="10985" max="10985" width="12.44140625" style="13" customWidth="1"/>
+    <col min="10986" max="10986" width="11.44140625" style="13" customWidth="1"/>
+    <col min="10987" max="10987" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="10988" max="10988" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="10989" max="10989" width="11.44140625" style="13" customWidth="1"/>
+    <col min="10990" max="10990" width="9.109375" style="13" customWidth="1"/>
+    <col min="10991" max="10992" width="10" style="13" customWidth="1"/>
+    <col min="10993" max="10993" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="10994" max="11231" width="8.88671875" style="13"/>
+    <col min="11232" max="11232" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="11233" max="11233" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="11234" max="11234" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="11235" max="11235" width="10" style="13" customWidth="1"/>
+    <col min="11236" max="11236" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="11237" max="11237" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="11238" max="11238" width="13.44140625" style="13" customWidth="1"/>
+    <col min="11239" max="11239" width="12.109375" style="13" customWidth="1"/>
+    <col min="11240" max="11240" width="11.88671875" style="13" customWidth="1"/>
+    <col min="11241" max="11241" width="12.44140625" style="13" customWidth="1"/>
+    <col min="11242" max="11242" width="11.44140625" style="13" customWidth="1"/>
+    <col min="11243" max="11243" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="11244" max="11244" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="11245" max="11245" width="11.44140625" style="13" customWidth="1"/>
+    <col min="11246" max="11246" width="9.109375" style="13" customWidth="1"/>
+    <col min="11247" max="11248" width="10" style="13" customWidth="1"/>
+    <col min="11249" max="11249" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="11250" max="11487" width="8.88671875" style="13"/>
+    <col min="11488" max="11488" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="11489" max="11489" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="11490" max="11490" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="11491" max="11491" width="10" style="13" customWidth="1"/>
+    <col min="11492" max="11492" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="11493" max="11493" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="11494" max="11494" width="13.44140625" style="13" customWidth="1"/>
+    <col min="11495" max="11495" width="12.109375" style="13" customWidth="1"/>
+    <col min="11496" max="11496" width="11.88671875" style="13" customWidth="1"/>
+    <col min="11497" max="11497" width="12.44140625" style="13" customWidth="1"/>
+    <col min="11498" max="11498" width="11.44140625" style="13" customWidth="1"/>
+    <col min="11499" max="11499" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="11500" max="11500" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="11501" max="11501" width="11.44140625" style="13" customWidth="1"/>
+    <col min="11502" max="11502" width="9.109375" style="13" customWidth="1"/>
+    <col min="11503" max="11504" width="10" style="13" customWidth="1"/>
+    <col min="11505" max="11505" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="11506" max="11743" width="8.88671875" style="13"/>
+    <col min="11744" max="11744" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="11745" max="11745" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="11746" max="11746" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="11747" max="11747" width="10" style="13" customWidth="1"/>
+    <col min="11748" max="11748" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="11749" max="11749" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="11750" max="11750" width="13.44140625" style="13" customWidth="1"/>
+    <col min="11751" max="11751" width="12.109375" style="13" customWidth="1"/>
+    <col min="11752" max="11752" width="11.88671875" style="13" customWidth="1"/>
+    <col min="11753" max="11753" width="12.44140625" style="13" customWidth="1"/>
+    <col min="11754" max="11754" width="11.44140625" style="13" customWidth="1"/>
+    <col min="11755" max="11755" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="11756" max="11756" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="11757" max="11757" width="11.44140625" style="13" customWidth="1"/>
+    <col min="11758" max="11758" width="9.109375" style="13" customWidth="1"/>
+    <col min="11759" max="11760" width="10" style="13" customWidth="1"/>
+    <col min="11761" max="11761" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="11762" max="11999" width="8.88671875" style="13"/>
+    <col min="12000" max="12000" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="12001" max="12001" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="12002" max="12002" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="12003" max="12003" width="10" style="13" customWidth="1"/>
+    <col min="12004" max="12004" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="12005" max="12005" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="12006" max="12006" width="13.44140625" style="13" customWidth="1"/>
+    <col min="12007" max="12007" width="12.109375" style="13" customWidth="1"/>
+    <col min="12008" max="12008" width="11.88671875" style="13" customWidth="1"/>
+    <col min="12009" max="12009" width="12.44140625" style="13" customWidth="1"/>
+    <col min="12010" max="12010" width="11.44140625" style="13" customWidth="1"/>
+    <col min="12011" max="12011" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="12012" max="12012" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="12013" max="12013" width="11.44140625" style="13" customWidth="1"/>
+    <col min="12014" max="12014" width="9.109375" style="13" customWidth="1"/>
+    <col min="12015" max="12016" width="10" style="13" customWidth="1"/>
+    <col min="12017" max="12017" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="12018" max="12255" width="8.88671875" style="13"/>
+    <col min="12256" max="12256" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="12257" max="12257" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="12258" max="12258" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="12259" max="12259" width="10" style="13" customWidth="1"/>
+    <col min="12260" max="12260" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="12261" max="12261" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="12262" max="12262" width="13.44140625" style="13" customWidth="1"/>
+    <col min="12263" max="12263" width="12.109375" style="13" customWidth="1"/>
+    <col min="12264" max="12264" width="11.88671875" style="13" customWidth="1"/>
+    <col min="12265" max="12265" width="12.44140625" style="13" customWidth="1"/>
+    <col min="12266" max="12266" width="11.44140625" style="13" customWidth="1"/>
+    <col min="12267" max="12267" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="12268" max="12268" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="12269" max="12269" width="11.44140625" style="13" customWidth="1"/>
+    <col min="12270" max="12270" width="9.109375" style="13" customWidth="1"/>
+    <col min="12271" max="12272" width="10" style="13" customWidth="1"/>
+    <col min="12273" max="12273" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="12274" max="12511" width="8.88671875" style="13"/>
+    <col min="12512" max="12512" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="12513" max="12513" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="12514" max="12514" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="12515" max="12515" width="10" style="13" customWidth="1"/>
+    <col min="12516" max="12516" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="12517" max="12517" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="12518" max="12518" width="13.44140625" style="13" customWidth="1"/>
+    <col min="12519" max="12519" width="12.109375" style="13" customWidth="1"/>
+    <col min="12520" max="12520" width="11.88671875" style="13" customWidth="1"/>
+    <col min="12521" max="12521" width="12.44140625" style="13" customWidth="1"/>
+    <col min="12522" max="12522" width="11.44140625" style="13" customWidth="1"/>
+    <col min="12523" max="12523" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="12524" max="12524" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="12525" max="12525" width="11.44140625" style="13" customWidth="1"/>
+    <col min="12526" max="12526" width="9.109375" style="13" customWidth="1"/>
+    <col min="12527" max="12528" width="10" style="13" customWidth="1"/>
+    <col min="12529" max="12529" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="12530" max="12767" width="8.88671875" style="13"/>
+    <col min="12768" max="12768" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="12769" max="12769" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="12770" max="12770" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="12771" max="12771" width="10" style="13" customWidth="1"/>
+    <col min="12772" max="12772" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="12773" max="12773" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="12774" max="12774" width="13.44140625" style="13" customWidth="1"/>
+    <col min="12775" max="12775" width="12.109375" style="13" customWidth="1"/>
+    <col min="12776" max="12776" width="11.88671875" style="13" customWidth="1"/>
+    <col min="12777" max="12777" width="12.44140625" style="13" customWidth="1"/>
+    <col min="12778" max="12778" width="11.44140625" style="13" customWidth="1"/>
+    <col min="12779" max="12779" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="12780" max="12780" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="12781" max="12781" width="11.44140625" style="13" customWidth="1"/>
+    <col min="12782" max="12782" width="9.109375" style="13" customWidth="1"/>
+    <col min="12783" max="12784" width="10" style="13" customWidth="1"/>
+    <col min="12785" max="12785" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="12786" max="13023" width="8.88671875" style="13"/>
+    <col min="13024" max="13024" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="13025" max="13025" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="13026" max="13026" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="13027" max="13027" width="10" style="13" customWidth="1"/>
+    <col min="13028" max="13028" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="13029" max="13029" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="13030" max="13030" width="13.44140625" style="13" customWidth="1"/>
+    <col min="13031" max="13031" width="12.109375" style="13" customWidth="1"/>
+    <col min="13032" max="13032" width="11.88671875" style="13" customWidth="1"/>
+    <col min="13033" max="13033" width="12.44140625" style="13" customWidth="1"/>
+    <col min="13034" max="13034" width="11.44140625" style="13" customWidth="1"/>
+    <col min="13035" max="13035" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="13036" max="13036" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="13037" max="13037" width="11.44140625" style="13" customWidth="1"/>
+    <col min="13038" max="13038" width="9.109375" style="13" customWidth="1"/>
+    <col min="13039" max="13040" width="10" style="13" customWidth="1"/>
+    <col min="13041" max="13041" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="13042" max="13279" width="8.88671875" style="13"/>
+    <col min="13280" max="13280" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="13281" max="13281" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="13282" max="13282" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="13283" max="13283" width="10" style="13" customWidth="1"/>
+    <col min="13284" max="13284" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="13285" max="13285" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="13286" max="13286" width="13.44140625" style="13" customWidth="1"/>
+    <col min="13287" max="13287" width="12.109375" style="13" customWidth="1"/>
+    <col min="13288" max="13288" width="11.88671875" style="13" customWidth="1"/>
+    <col min="13289" max="13289" width="12.44140625" style="13" customWidth="1"/>
+    <col min="13290" max="13290" width="11.44140625" style="13" customWidth="1"/>
+    <col min="13291" max="13291" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="13292" max="13292" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="13293" max="13293" width="11.44140625" style="13" customWidth="1"/>
+    <col min="13294" max="13294" width="9.109375" style="13" customWidth="1"/>
+    <col min="13295" max="13296" width="10" style="13" customWidth="1"/>
+    <col min="13297" max="13297" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="13298" max="13535" width="8.88671875" style="13"/>
+    <col min="13536" max="13536" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="13537" max="13537" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="13538" max="13538" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="13539" max="13539" width="10" style="13" customWidth="1"/>
+    <col min="13540" max="13540" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="13541" max="13541" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="13542" max="13542" width="13.44140625" style="13" customWidth="1"/>
+    <col min="13543" max="13543" width="12.109375" style="13" customWidth="1"/>
+    <col min="13544" max="13544" width="11.88671875" style="13" customWidth="1"/>
+    <col min="13545" max="13545" width="12.44140625" style="13" customWidth="1"/>
+    <col min="13546" max="13546" width="11.44140625" style="13" customWidth="1"/>
+    <col min="13547" max="13547" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="13548" max="13548" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="13549" max="13549" width="11.44140625" style="13" customWidth="1"/>
+    <col min="13550" max="13550" width="9.109375" style="13" customWidth="1"/>
+    <col min="13551" max="13552" width="10" style="13" customWidth="1"/>
+    <col min="13553" max="13553" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="13554" max="13791" width="8.88671875" style="13"/>
+    <col min="13792" max="13792" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="13793" max="13793" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="13794" max="13794" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="13795" max="13795" width="10" style="13" customWidth="1"/>
+    <col min="13796" max="13796" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="13797" max="13797" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="13798" max="13798" width="13.44140625" style="13" customWidth="1"/>
+    <col min="13799" max="13799" width="12.109375" style="13" customWidth="1"/>
+    <col min="13800" max="13800" width="11.88671875" style="13" customWidth="1"/>
+    <col min="13801" max="13801" width="12.44140625" style="13" customWidth="1"/>
+    <col min="13802" max="13802" width="11.44140625" style="13" customWidth="1"/>
+    <col min="13803" max="13803" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="13804" max="13804" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="13805" max="13805" width="11.44140625" style="13" customWidth="1"/>
+    <col min="13806" max="13806" width="9.109375" style="13" customWidth="1"/>
+    <col min="13807" max="13808" width="10" style="13" customWidth="1"/>
+    <col min="13809" max="13809" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="13810" max="14047" width="8.88671875" style="13"/>
+    <col min="14048" max="14048" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="14049" max="14049" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="14050" max="14050" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="14051" max="14051" width="10" style="13" customWidth="1"/>
+    <col min="14052" max="14052" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="14053" max="14053" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="14054" max="14054" width="13.44140625" style="13" customWidth="1"/>
+    <col min="14055" max="14055" width="12.109375" style="13" customWidth="1"/>
+    <col min="14056" max="14056" width="11.88671875" style="13" customWidth="1"/>
+    <col min="14057" max="14057" width="12.44140625" style="13" customWidth="1"/>
+    <col min="14058" max="14058" width="11.44140625" style="13" customWidth="1"/>
+    <col min="14059" max="14059" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="14060" max="14060" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="14061" max="14061" width="11.44140625" style="13" customWidth="1"/>
+    <col min="14062" max="14062" width="9.109375" style="13" customWidth="1"/>
+    <col min="14063" max="14064" width="10" style="13" customWidth="1"/>
+    <col min="14065" max="14065" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="14066" max="14303" width="8.88671875" style="13"/>
+    <col min="14304" max="14304" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="14305" max="14305" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="14306" max="14306" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="14307" max="14307" width="10" style="13" customWidth="1"/>
+    <col min="14308" max="14308" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="14309" max="14309" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="14310" max="14310" width="13.44140625" style="13" customWidth="1"/>
+    <col min="14311" max="14311" width="12.109375" style="13" customWidth="1"/>
+    <col min="14312" max="14312" width="11.88671875" style="13" customWidth="1"/>
+    <col min="14313" max="14313" width="12.44140625" style="13" customWidth="1"/>
+    <col min="14314" max="14314" width="11.44140625" style="13" customWidth="1"/>
+    <col min="14315" max="14315" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="14316" max="14316" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="14317" max="14317" width="11.44140625" style="13" customWidth="1"/>
+    <col min="14318" max="14318" width="9.109375" style="13" customWidth="1"/>
+    <col min="14319" max="14320" width="10" style="13" customWidth="1"/>
+    <col min="14321" max="14321" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="14322" max="14559" width="8.88671875" style="13"/>
+    <col min="14560" max="14560" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="14561" max="14561" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="14562" max="14562" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="14563" max="14563" width="10" style="13" customWidth="1"/>
+    <col min="14564" max="14564" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="14565" max="14565" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="14566" max="14566" width="13.44140625" style="13" customWidth="1"/>
+    <col min="14567" max="14567" width="12.109375" style="13" customWidth="1"/>
+    <col min="14568" max="14568" width="11.88671875" style="13" customWidth="1"/>
+    <col min="14569" max="14569" width="12.44140625" style="13" customWidth="1"/>
+    <col min="14570" max="14570" width="11.44140625" style="13" customWidth="1"/>
+    <col min="14571" max="14571" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="14572" max="14572" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="14573" max="14573" width="11.44140625" style="13" customWidth="1"/>
+    <col min="14574" max="14574" width="9.109375" style="13" customWidth="1"/>
+    <col min="14575" max="14576" width="10" style="13" customWidth="1"/>
+    <col min="14577" max="14577" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="14578" max="14815" width="8.88671875" style="13"/>
+    <col min="14816" max="14816" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="14817" max="14817" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="14818" max="14818" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="14819" max="14819" width="10" style="13" customWidth="1"/>
+    <col min="14820" max="14820" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="14821" max="14821" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="14822" max="14822" width="13.44140625" style="13" customWidth="1"/>
+    <col min="14823" max="14823" width="12.109375" style="13" customWidth="1"/>
+    <col min="14824" max="14824" width="11.88671875" style="13" customWidth="1"/>
+    <col min="14825" max="14825" width="12.44140625" style="13" customWidth="1"/>
+    <col min="14826" max="14826" width="11.44140625" style="13" customWidth="1"/>
+    <col min="14827" max="14827" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="14828" max="14828" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="14829" max="14829" width="11.44140625" style="13" customWidth="1"/>
+    <col min="14830" max="14830" width="9.109375" style="13" customWidth="1"/>
+    <col min="14831" max="14832" width="10" style="13" customWidth="1"/>
+    <col min="14833" max="14833" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="14834" max="15071" width="8.88671875" style="13"/>
+    <col min="15072" max="15072" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="15073" max="15073" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="15074" max="15074" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="15075" max="15075" width="10" style="13" customWidth="1"/>
+    <col min="15076" max="15076" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="15077" max="15077" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="15078" max="15078" width="13.44140625" style="13" customWidth="1"/>
+    <col min="15079" max="15079" width="12.109375" style="13" customWidth="1"/>
+    <col min="15080" max="15080" width="11.88671875" style="13" customWidth="1"/>
+    <col min="15081" max="15081" width="12.44140625" style="13" customWidth="1"/>
+    <col min="15082" max="15082" width="11.44140625" style="13" customWidth="1"/>
+    <col min="15083" max="15083" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="15084" max="15084" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="15085" max="15085" width="11.44140625" style="13" customWidth="1"/>
+    <col min="15086" max="15086" width="9.109375" style="13" customWidth="1"/>
+    <col min="15087" max="15088" width="10" style="13" customWidth="1"/>
+    <col min="15089" max="15089" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="15090" max="15327" width="8.88671875" style="13"/>
+    <col min="15328" max="15328" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="15329" max="15329" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="15330" max="15330" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="15331" max="15331" width="10" style="13" customWidth="1"/>
+    <col min="15332" max="15332" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="15333" max="15333" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="15334" max="15334" width="13.44140625" style="13" customWidth="1"/>
+    <col min="15335" max="15335" width="12.109375" style="13" customWidth="1"/>
+    <col min="15336" max="15336" width="11.88671875" style="13" customWidth="1"/>
+    <col min="15337" max="15337" width="12.44140625" style="13" customWidth="1"/>
+    <col min="15338" max="15338" width="11.44140625" style="13" customWidth="1"/>
+    <col min="15339" max="15339" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="15340" max="15340" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="15341" max="15341" width="11.44140625" style="13" customWidth="1"/>
+    <col min="15342" max="15342" width="9.109375" style="13" customWidth="1"/>
+    <col min="15343" max="15344" width="10" style="13" customWidth="1"/>
+    <col min="15345" max="15345" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="15346" max="15583" width="8.88671875" style="13"/>
+    <col min="15584" max="15584" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="15585" max="15585" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="15586" max="15586" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="15587" max="15587" width="10" style="13" customWidth="1"/>
+    <col min="15588" max="15588" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="15589" max="15589" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="15590" max="15590" width="13.44140625" style="13" customWidth="1"/>
+    <col min="15591" max="15591" width="12.109375" style="13" customWidth="1"/>
+    <col min="15592" max="15592" width="11.88671875" style="13" customWidth="1"/>
+    <col min="15593" max="15593" width="12.44140625" style="13" customWidth="1"/>
+    <col min="15594" max="15594" width="11.44140625" style="13" customWidth="1"/>
+    <col min="15595" max="15595" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="15596" max="15596" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="15597" max="15597" width="11.44140625" style="13" customWidth="1"/>
+    <col min="15598" max="15598" width="9.109375" style="13" customWidth="1"/>
+    <col min="15599" max="15600" width="10" style="13" customWidth="1"/>
+    <col min="15601" max="15601" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="15602" max="15839" width="8.88671875" style="13"/>
+    <col min="15840" max="15840" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="15841" max="15841" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="15842" max="15842" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="15843" max="15843" width="10" style="13" customWidth="1"/>
+    <col min="15844" max="15844" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="15845" max="15845" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="15846" max="15846" width="13.44140625" style="13" customWidth="1"/>
+    <col min="15847" max="15847" width="12.109375" style="13" customWidth="1"/>
+    <col min="15848" max="15848" width="11.88671875" style="13" customWidth="1"/>
+    <col min="15849" max="15849" width="12.44140625" style="13" customWidth="1"/>
+    <col min="15850" max="15850" width="11.44140625" style="13" customWidth="1"/>
+    <col min="15851" max="15851" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="15852" max="15852" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="15853" max="15853" width="11.44140625" style="13" customWidth="1"/>
+    <col min="15854" max="15854" width="9.109375" style="13" customWidth="1"/>
+    <col min="15855" max="15856" width="10" style="13" customWidth="1"/>
+    <col min="15857" max="15857" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="15858" max="16095" width="8.88671875" style="13"/>
+    <col min="16096" max="16096" width="66.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="16097" max="16097" width="11.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="16098" max="16098" width="8.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="16099" max="16099" width="10" style="13" customWidth="1"/>
+    <col min="16100" max="16100" width="12.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="16101" max="16101" width="13.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="16102" max="16102" width="13.44140625" style="13" customWidth="1"/>
+    <col min="16103" max="16103" width="12.109375" style="13" customWidth="1"/>
+    <col min="16104" max="16104" width="11.88671875" style="13" customWidth="1"/>
+    <col min="16105" max="16105" width="12.44140625" style="13" customWidth="1"/>
+    <col min="16106" max="16106" width="11.44140625" style="13" customWidth="1"/>
+    <col min="16107" max="16107" width="13.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="16108" max="16108" width="9.5546875" style="13" bestFit="1" customWidth="1"/>
+    <col min="16109" max="16109" width="11.44140625" style="13" customWidth="1"/>
+    <col min="16110" max="16110" width="9.109375" style="13" customWidth="1"/>
+    <col min="16111" max="16112" width="10" style="13" customWidth="1"/>
+    <col min="16113" max="16113" width="10.88671875" style="13" bestFit="1" customWidth="1"/>
+    <col min="16114" max="16384" width="8.88671875" style="13"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B1" s="55">
+        <v>44835</v>
+      </c>
+      <c r="C1" s="55">
+        <v>44927</v>
+      </c>
+      <c r="D1" s="55">
+        <v>45017</v>
+      </c>
+      <c r="E1" s="55">
+        <v>45108</v>
+      </c>
+      <c r="F1" s="55">
+        <v>45200</v>
+      </c>
+      <c r="G1" s="55">
+        <v>45292</v>
+      </c>
+      <c r="H1" s="55">
+        <v>45383</v>
+      </c>
+      <c r="I1" s="55">
+        <v>45474</v>
+      </c>
+      <c r="J1" s="55">
+        <v>45566</v>
+      </c>
+      <c r="K1" s="55">
+        <v>45658</v>
+      </c>
+      <c r="L1" s="55">
+        <v>45748</v>
+      </c>
+      <c r="M1" s="55">
+        <v>45839</v>
+      </c>
+      <c r="N1" s="55">
+        <v>45931</v>
+      </c>
+      <c r="O1" s="55">
+        <v>46023</v>
+      </c>
+      <c r="P1" s="55">
+        <v>46113</v>
+      </c>
+      <c r="Q1" s="55">
+        <v>46204</v>
+      </c>
+      <c r="R1" s="55">
+        <v>46296</v>
+      </c>
+      <c r="S1" s="55">
+        <v>46388</v>
+      </c>
+      <c r="T1" s="55">
+        <v>46478</v>
+      </c>
+      <c r="U1" s="55">
+        <v>46569</v>
+      </c>
+      <c r="V1" s="55">
+        <v>46661</v>
+      </c>
+      <c r="W1" s="55">
+        <v>46753</v>
+      </c>
+      <c r="X1" s="55">
+        <v>46844</v>
+      </c>
+      <c r="Y1" s="55">
+        <v>46935</v>
+      </c>
+      <c r="Z1" s="55">
+        <v>47027</v>
+      </c>
+    </row>
+    <row r="2" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="A2" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="B2" s="42">
+        <v>5297</v>
+      </c>
+      <c r="C2" s="42">
+        <v>9007.3539842835198</v>
+      </c>
+      <c r="D2" s="42">
+        <v>970.11401264363667</v>
+      </c>
+      <c r="E2" s="42">
+        <v>69128.378897873175</v>
+      </c>
+      <c r="F2" s="42">
+        <v>61973.066677937182</v>
+      </c>
+      <c r="G2" s="42">
+        <v>3377.1198957684828</v>
+      </c>
+      <c r="H2" s="42">
+        <v>3199.7224747239125</v>
+      </c>
+      <c r="I2" s="42">
+        <v>36410.411294655423</v>
+      </c>
+      <c r="J2" s="42">
+        <v>9217.3930356614001</v>
+      </c>
+      <c r="K2" s="42">
+        <v>49978.599445284752</v>
+      </c>
+      <c r="L2" s="42">
+        <v>32938.589097162141</v>
+      </c>
+      <c r="M2" s="42">
+        <v>51467.687001131359</v>
+      </c>
+      <c r="N2" s="42">
+        <v>106260.36872833429</v>
+      </c>
+      <c r="O2" s="42">
+        <v>0</v>
+      </c>
+      <c r="P2" s="42">
+        <f t="shared" ref="P2:Z2" ca="1" si="0">O2*(RAND()*(1.04-1.025)+1.025)</f>
+        <v>0</v>
+      </c>
+      <c r="Q2" s="42">
+        <f t="shared" ca="1" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="R2" s="42">
+        <f t="shared" ca="1" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="S2" s="42">
+        <f t="shared" ca="1" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="T2" s="42">
+        <f t="shared" ca="1" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="U2" s="42">
+        <f t="shared" ca="1" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="V2" s="42">
+        <f t="shared" ca="1" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="W2" s="42">
+        <f t="shared" ca="1" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="X2" s="42">
+        <f t="shared" ca="1" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="Y2" s="42">
+        <f t="shared" ca="1" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="Z2" s="42">
+        <f t="shared" ca="1" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="A3" s="12" t="s">
+        <v>83</v>
+      </c>
+      <c r="B3" s="42">
+        <v>109164.73109594014</v>
+      </c>
+      <c r="C3" s="42">
+        <v>109364.8</v>
+      </c>
+      <c r="D3" s="42">
+        <v>104862.03127593001</v>
+      </c>
+      <c r="E3" s="42">
+        <v>107460.70783204175</v>
+      </c>
+      <c r="F3" s="42">
+        <v>144869.31134359751</v>
+      </c>
+      <c r="G3" s="42">
+        <v>158085.8680208546</v>
+      </c>
+      <c r="H3" s="42">
+        <v>128120.81252859323</v>
+      </c>
+      <c r="I3" s="42">
+        <v>110365.99498029456</v>
+      </c>
+      <c r="J3" s="42">
+        <v>100237.62176769711</v>
+      </c>
+      <c r="K3" s="42">
+        <v>143107.0116076436</v>
+      </c>
+      <c r="L3" s="42">
+        <v>154871.78207848271</v>
+      </c>
+      <c r="M3" s="42">
+        <v>149712.56572213367</v>
+      </c>
+      <c r="N3" s="42">
+        <v>150175.74565049403</v>
+      </c>
+      <c r="O3" s="42">
+        <v>0</v>
+      </c>
+      <c r="P3" s="42">
+        <f t="shared" ref="P3:Z4" ca="1" si="1">O3*(RAND()*(1.15-0.93)+0.93)</f>
+        <v>0</v>
+      </c>
+      <c r="Q3" s="42">
+        <f t="shared" ca="1" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="R3" s="42">
+        <f t="shared" ca="1" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="S3" s="42">
+        <f t="shared" ca="1" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="T3" s="42">
+        <f t="shared" ca="1" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="U3" s="42">
+        <f t="shared" ca="1" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="V3" s="42">
+        <f t="shared" ca="1" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="W3" s="42">
+        <f t="shared" ca="1" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="X3" s="42">
+        <f t="shared" ca="1" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y3" s="42">
+        <f t="shared" ca="1" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Z3" s="42">
+        <f t="shared" ca="1" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="A4" s="12" t="s">
+        <v>84</v>
+      </c>
+      <c r="B4" s="42">
+        <v>168142.95269518925</v>
+      </c>
+      <c r="C4" s="42">
+        <v>176213.3910344794</v>
+      </c>
+      <c r="D4" s="42">
+        <v>183797.04964974552</v>
+      </c>
+      <c r="E4" s="42">
+        <v>188097.33499598625</v>
+      </c>
+      <c r="F4" s="42">
+        <v>195169.87089099811</v>
+      </c>
+      <c r="G4" s="42">
+        <v>205630.11959630589</v>
+      </c>
+      <c r="H4" s="42">
+        <v>219371.7267897749</v>
+      </c>
+      <c r="I4" s="42">
+        <v>213132.14646400703</v>
+      </c>
+      <c r="J4" s="42">
+        <v>226775.31416633673</v>
+      </c>
+      <c r="K4" s="42">
+        <v>238177.54703184307</v>
+      </c>
+      <c r="L4" s="42">
+        <v>253364.29098184008</v>
+      </c>
+      <c r="M4" s="42">
+        <v>245838.12279105405</v>
+      </c>
+      <c r="N4" s="42">
+        <v>262120.26923055129</v>
+      </c>
+      <c r="O4" s="42">
+        <v>0</v>
+      </c>
+      <c r="P4" s="42">
+        <f t="shared" ca="1" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Q4" s="42">
+        <f t="shared" ca="1" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="R4" s="42">
+        <f t="shared" ca="1" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="S4" s="42">
+        <f t="shared" ca="1" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="T4" s="42">
+        <f t="shared" ca="1" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="U4" s="42">
+        <f t="shared" ca="1" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="V4" s="42">
+        <f t="shared" ca="1" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="W4" s="42">
+        <f t="shared" ca="1" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="X4" s="42">
+        <f t="shared" ca="1" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y4" s="42">
+        <f t="shared" ca="1" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Z4" s="42">
+        <f t="shared" ca="1" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="A5" s="12" t="s">
+        <v>85</v>
+      </c>
+      <c r="B5" s="42">
+        <v>0</v>
+      </c>
+      <c r="C5" s="42">
+        <v>0</v>
+      </c>
+      <c r="D5" s="42">
+        <v>0</v>
+      </c>
+      <c r="E5" s="42">
+        <v>0</v>
+      </c>
+      <c r="F5" s="42">
+        <v>0</v>
+      </c>
+      <c r="G5" s="42">
+        <v>0</v>
+      </c>
+      <c r="H5" s="42">
+        <v>0</v>
+      </c>
+      <c r="I5" s="42">
+        <v>0</v>
+      </c>
+      <c r="J5" s="42">
+        <v>0</v>
+      </c>
+      <c r="K5" s="42">
+        <v>0</v>
+      </c>
+      <c r="L5" s="42">
+        <v>0</v>
+      </c>
+      <c r="M5" s="42">
+        <v>0</v>
+      </c>
+      <c r="N5" s="95">
+        <v>0</v>
+      </c>
+      <c r="O5" s="42">
+        <v>0</v>
+      </c>
+      <c r="P5" s="42">
+        <f t="shared" ref="P5:Z5" ca="1" si="2">O5*(RAND()*(1.05-1.1)+1.05)</f>
+        <v>0</v>
+      </c>
+      <c r="Q5" s="42">
+        <f t="shared" ca="1" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="R5" s="42">
+        <f t="shared" ca="1" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="S5" s="42">
+        <f t="shared" ca="1" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="T5" s="42">
+        <f t="shared" ca="1" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="U5" s="42">
+        <f t="shared" ca="1" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="V5" s="42">
+        <f t="shared" ca="1" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="W5" s="42">
+        <f t="shared" ca="1" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="X5" s="42">
+        <f t="shared" ca="1" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="Y5" s="42">
+        <f t="shared" ca="1" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="Z5" s="42">
+        <f t="shared" ca="1" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="A6" s="12" t="s">
+        <v>86</v>
+      </c>
+      <c r="B6" s="42">
+        <f>SUM(B2:B5)</f>
+        <v>282604.68379112938</v>
+      </c>
+      <c r="C6" s="42">
+        <f t="shared" ref="C6:N6" si="3">SUM(C2:C5)</f>
+        <v>294585.54501876293</v>
+      </c>
+      <c r="D6" s="42">
+        <f t="shared" si="3"/>
+        <v>289629.19493831915</v>
+      </c>
+      <c r="E6" s="42">
+        <f t="shared" si="3"/>
+        <v>364686.42172590119</v>
+      </c>
+      <c r="F6" s="42">
+        <f t="shared" si="3"/>
+        <v>402012.24891253281</v>
+      </c>
+      <c r="G6" s="42">
+        <f t="shared" si="3"/>
+        <v>367093.10751292895</v>
+      </c>
+      <c r="H6" s="42">
+        <f t="shared" si="3"/>
+        <v>350692.26179309201</v>
+      </c>
+      <c r="I6" s="42">
+        <f t="shared" si="3"/>
+        <v>359908.55273895699</v>
+      </c>
+      <c r="J6" s="42">
+        <f t="shared" si="3"/>
+        <v>336230.32896969526</v>
+      </c>
+      <c r="K6" s="42">
+        <f t="shared" si="3"/>
+        <v>431263.15808477142</v>
+      </c>
+      <c r="L6" s="42">
+        <f t="shared" si="3"/>
+        <v>441174.66215748491</v>
+      </c>
+      <c r="M6" s="42">
+        <f t="shared" si="3"/>
+        <v>447018.37551431905</v>
+      </c>
+      <c r="N6" s="42">
+        <f t="shared" si="3"/>
+        <v>518556.38360937964</v>
+      </c>
+      <c r="O6" s="42">
+        <v>0</v>
+      </c>
+      <c r="P6" s="42">
+        <f t="shared" ref="P6:Z6" ca="1" si="4">O6*(RAND()*(1.05-1.01)+1.01)</f>
+        <v>0</v>
+      </c>
+      <c r="Q6" s="42">
+        <f t="shared" ca="1" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="R6" s="42">
+        <f t="shared" ca="1" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="S6" s="42">
+        <f t="shared" ca="1" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="T6" s="42">
+        <f t="shared" ca="1" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="U6" s="42">
+        <f t="shared" ca="1" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="V6" s="42">
+        <f t="shared" ca="1" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="W6" s="42">
+        <f t="shared" ca="1" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="X6" s="42">
+        <f t="shared" ca="1" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Y6" s="42">
+        <f t="shared" ca="1" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="Z6" s="42">
+        <f t="shared" ca="1" si="4"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="A7" s="12" t="s">
+        <v>87</v>
+      </c>
+      <c r="B7" s="42">
+        <v>874825.43239509477</v>
+      </c>
+      <c r="C7" s="42">
+        <v>888977.78041387827</v>
+      </c>
+      <c r="D7" s="42">
+        <v>898941.57135464589</v>
+      </c>
+      <c r="E7" s="42">
+        <v>907807.36364481726</v>
+      </c>
+      <c r="F7" s="42">
+        <v>966197.85825326247</v>
+      </c>
+      <c r="G7" s="42">
+        <v>1017923.093222491</v>
+      </c>
+      <c r="H7" s="42">
+        <v>1059865.8224482499</v>
+      </c>
+      <c r="I7" s="42">
+        <v>1131525.9128823632</v>
+      </c>
+      <c r="J7" s="42">
+        <v>1158386.8243463556</v>
+      </c>
+      <c r="K7" s="42">
+        <v>1159324.9760359023</v>
+      </c>
+      <c r="L7" s="42">
+        <v>1163625.9721146177</v>
+      </c>
+      <c r="M7" s="42">
+        <v>1165859.866725384</v>
+      </c>
+      <c r="N7" s="42">
+        <v>1166156.1778461398</v>
+      </c>
+      <c r="O7" s="42">
+        <v>0</v>
+      </c>
+      <c r="P7" s="42">
+        <v>0</v>
+      </c>
+      <c r="Q7" s="42">
+        <v>0</v>
+      </c>
+      <c r="R7" s="42">
+        <v>0</v>
+      </c>
+      <c r="S7" s="42">
+        <v>0</v>
+      </c>
+      <c r="T7" s="42">
+        <v>0</v>
+      </c>
+      <c r="U7" s="42">
+        <v>0</v>
+      </c>
+      <c r="V7" s="42">
+        <v>0</v>
+      </c>
+      <c r="W7" s="42">
+        <v>0</v>
+      </c>
+      <c r="X7" s="42">
+        <v>0</v>
+      </c>
+      <c r="Y7" s="42">
+        <v>0</v>
+      </c>
+      <c r="Z7" s="42">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="A8" s="12" t="s">
+        <v>88</v>
+      </c>
+      <c r="B8" s="42">
+        <v>0</v>
+      </c>
+      <c r="C8" s="42">
+        <v>0</v>
+      </c>
+      <c r="D8" s="42">
+        <v>0</v>
+      </c>
+      <c r="E8" s="42">
+        <v>0</v>
+      </c>
+      <c r="F8" s="42">
+        <v>0</v>
+      </c>
+      <c r="G8" s="42">
+        <v>0</v>
+      </c>
+      <c r="H8" s="42">
+        <v>0</v>
+      </c>
+      <c r="I8" s="42">
+        <v>0</v>
+      </c>
+      <c r="J8" s="42">
+        <v>0</v>
+      </c>
+      <c r="K8" s="42">
+        <v>0</v>
+      </c>
+      <c r="L8" s="42">
+        <v>0</v>
+      </c>
+      <c r="M8" s="42">
+        <v>0</v>
+      </c>
+      <c r="N8" s="42">
+        <v>0</v>
+      </c>
+      <c r="O8" s="42">
+        <v>0</v>
+      </c>
+      <c r="P8" s="42">
+        <f t="shared" ref="P8:Z8" ca="1" si="5">O8*(RAND()*(1.04-1.025)+1.025)</f>
+        <v>0</v>
+      </c>
+      <c r="Q8" s="42">
+        <f t="shared" ca="1" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="R8" s="42">
+        <f t="shared" ca="1" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="S8" s="42">
+        <f t="shared" ca="1" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="T8" s="42">
+        <f t="shared" ca="1" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="U8" s="42">
+        <f t="shared" ca="1" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="V8" s="42">
+        <f t="shared" ca="1" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="W8" s="42">
+        <f t="shared" ca="1" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="X8" s="42">
+        <f t="shared" ca="1" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="Y8" s="42">
+        <f t="shared" ca="1" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="Z8" s="42">
+        <f t="shared" ca="1" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="A9" s="12" t="s">
+        <v>89</v>
+      </c>
+      <c r="B9" s="42">
+        <f>B6+B7+B8</f>
+        <v>1157430.1161862242</v>
+      </c>
+      <c r="C9" s="42">
+        <f t="shared" ref="C9:N9" si="6">C6+C7+C8</f>
+        <v>1183563.3254326412</v>
+      </c>
+      <c r="D9" s="42">
+        <f t="shared" si="6"/>
+        <v>1188570.766292965</v>
+      </c>
+      <c r="E9" s="42">
+        <f t="shared" si="6"/>
+        <v>1272493.7853707185</v>
+      </c>
+      <c r="F9" s="42">
+        <f t="shared" si="6"/>
+        <v>1368210.1071657953</v>
+      </c>
+      <c r="G9" s="42">
+        <f t="shared" si="6"/>
+        <v>1385016.20073542</v>
+      </c>
+      <c r="H9" s="42">
+        <f t="shared" si="6"/>
+        <v>1410558.0842413418</v>
+      </c>
+      <c r="I9" s="42">
+        <f t="shared" si="6"/>
+        <v>1491434.4656213201</v>
+      </c>
+      <c r="J9" s="42">
+        <f t="shared" si="6"/>
+        <v>1494617.1533160508</v>
+      </c>
+      <c r="K9" s="42">
+        <f t="shared" si="6"/>
+        <v>1590588.1341206736</v>
+      </c>
+      <c r="L9" s="42">
+        <f t="shared" si="6"/>
+        <v>1604800.6342721027</v>
+      </c>
+      <c r="M9" s="42">
+        <f t="shared" si="6"/>
+        <v>1612878.242239703</v>
+      </c>
+      <c r="N9" s="42">
+        <f t="shared" si="6"/>
+        <v>1684712.5614555194</v>
+      </c>
+      <c r="O9" s="42">
+        <f>'Cash Flow Statement_Actual'!O3*0.003</f>
+        <v>0</v>
+      </c>
+      <c r="P9" s="42">
+        <f>'Cash Flow Statement_Actual'!P3*0.003</f>
+        <v>0</v>
+      </c>
+      <c r="Q9" s="42">
+        <f>'Cash Flow Statement_Actual'!Q3*0.003</f>
+        <v>0</v>
+      </c>
+      <c r="R9" s="42">
+        <f>'Cash Flow Statement_Actual'!R3*0.003</f>
+        <v>0</v>
+      </c>
+      <c r="S9" s="42">
+        <f>'Cash Flow Statement_Actual'!S3*0.003</f>
+        <v>0</v>
+      </c>
+      <c r="T9" s="42">
+        <f>'Cash Flow Statement_Actual'!T3*0.003</f>
+        <v>0</v>
+      </c>
+      <c r="U9" s="42">
+        <f>'Cash Flow Statement_Actual'!U3*0.003</f>
+        <v>0</v>
+      </c>
+      <c r="V9" s="42">
+        <f>'Cash Flow Statement_Actual'!V3*0.003</f>
+        <v>0</v>
+      </c>
+      <c r="W9" s="42">
+        <f>'Cash Flow Statement_Actual'!W3*0.003</f>
+        <v>0</v>
+      </c>
+      <c r="X9" s="42">
+        <f>'Cash Flow Statement_Actual'!X3*0.003</f>
+        <v>0</v>
+      </c>
+      <c r="Y9" s="42">
+        <f>'Cash Flow Statement_Actual'!Y3*0.003</f>
+        <v>0</v>
+      </c>
+      <c r="Z9" s="42">
+        <f>'Cash Flow Statement_Actual'!Z3*0.003</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="A10" s="12" t="s">
+        <v>90</v>
+      </c>
+      <c r="B10" s="42">
+        <f>'Debt Schedule_Actual'!B5</f>
+        <v>0</v>
+      </c>
+      <c r="C10" s="42">
+        <f>'Debt Schedule_Actual'!C5</f>
+        <v>12000</v>
+      </c>
+      <c r="D10" s="42">
+        <f>'Debt Schedule_Actual'!D5</f>
+        <v>0</v>
+      </c>
+      <c r="E10" s="42">
+        <f>'Debt Schedule_Actual'!E5</f>
+        <v>0</v>
+      </c>
+      <c r="F10" s="42">
+        <f>'Debt Schedule_Actual'!F5</f>
+        <v>2000</v>
+      </c>
+      <c r="G10" s="42">
+        <f>'Debt Schedule_Actual'!G5</f>
+        <v>24000</v>
+      </c>
+      <c r="H10" s="42">
+        <f>'Debt Schedule_Actual'!H5</f>
+        <v>28000</v>
+      </c>
+      <c r="I10" s="42">
+        <f>'Debt Schedule_Actual'!I5</f>
+        <v>42000</v>
+      </c>
+      <c r="J10" s="42">
+        <f>'Debt Schedule_Actual'!J5</f>
+        <v>42000</v>
+      </c>
+      <c r="K10" s="42">
+        <f>'Debt Schedule_Actual'!K5</f>
+        <v>32000</v>
+      </c>
+      <c r="L10" s="42">
+        <f>'Debt Schedule_Actual'!L5</f>
+        <v>0</v>
+      </c>
+      <c r="M10" s="42">
+        <f>'Debt Schedule_Actual'!M5</f>
+        <v>0</v>
+      </c>
+      <c r="N10" s="42">
+        <f>'Debt Schedule_Actual'!N5</f>
+        <v>0</v>
+      </c>
+      <c r="O10" s="42">
+        <v>0</v>
+      </c>
+      <c r="P10" s="42">
+        <f t="shared" ref="P10:Z10" ca="1" si="7">O10*(RAND()*(1.04-1.025)+1.025)</f>
+        <v>0</v>
+      </c>
+      <c r="Q10" s="42">
+        <f t="shared" ca="1" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="R10" s="42">
+        <f t="shared" ca="1" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="S10" s="42">
+        <f t="shared" ca="1" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="T10" s="42">
+        <f t="shared" ca="1" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="U10" s="42">
+        <f t="shared" ca="1" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="V10" s="42">
+        <f t="shared" ca="1" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="W10" s="42">
+        <f t="shared" ca="1" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="X10" s="42">
+        <f t="shared" ca="1" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="Y10" s="42">
+        <f t="shared" ca="1" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="Z10" s="42">
+        <f t="shared" ca="1" si="7"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="A11" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="B11" s="42">
+        <v>0</v>
+      </c>
+      <c r="C11" s="42">
+        <v>0</v>
+      </c>
+      <c r="D11" s="42">
+        <v>0</v>
+      </c>
+      <c r="E11" s="42">
+        <v>0</v>
+      </c>
+      <c r="F11" s="42">
+        <v>0</v>
+      </c>
+      <c r="G11" s="42">
+        <v>0</v>
+      </c>
+      <c r="H11" s="42">
+        <v>0</v>
+      </c>
+      <c r="I11" s="42">
+        <v>0</v>
+      </c>
+      <c r="J11" s="42">
+        <v>0</v>
+      </c>
+      <c r="K11" s="42">
+        <v>0</v>
+      </c>
+      <c r="L11" s="42">
+        <v>0</v>
+      </c>
+      <c r="M11" s="42">
+        <v>0</v>
+      </c>
+      <c r="N11" s="42">
+        <v>0</v>
+      </c>
+      <c r="O11" s="42">
+        <v>0</v>
+      </c>
+      <c r="P11" s="42">
+        <v>0</v>
+      </c>
+      <c r="Q11" s="42">
+        <v>0</v>
+      </c>
+      <c r="R11" s="42">
+        <v>0</v>
+      </c>
+      <c r="S11" s="42">
+        <v>0</v>
+      </c>
+      <c r="T11" s="42">
+        <v>0</v>
+      </c>
+      <c r="U11" s="42">
+        <v>0</v>
+      </c>
+      <c r="V11" s="42">
+        <v>0</v>
+      </c>
+      <c r="W11" s="42">
+        <v>0</v>
+      </c>
+      <c r="X11" s="42">
+        <v>0</v>
+      </c>
+      <c r="Y11" s="42">
+        <v>0</v>
+      </c>
+      <c r="Z11" s="42">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="A12" s="12" t="s">
+        <v>92</v>
+      </c>
+      <c r="B12" s="42">
+        <f>'Working Capital_Actual'!B4</f>
+        <v>54982.535294664027</v>
+      </c>
+      <c r="C12" s="42">
+        <f>'Working Capital_Actual'!C4</f>
+        <v>21185.389800667006</v>
+      </c>
+      <c r="D12" s="42">
+        <f>'Working Capital_Actual'!D4</f>
+        <v>49077.648605494804</v>
+      </c>
+      <c r="E12" s="42">
+        <f>'Working Capital_Actual'!E4</f>
+        <v>6967.9673967445342</v>
+      </c>
+      <c r="F12" s="42">
+        <f>'Working Capital_Actual'!F4</f>
+        <v>20990.427847235434</v>
+      </c>
+      <c r="G12" s="42">
+        <f>'Working Capital_Actual'!G4</f>
+        <v>34687.193398158517</v>
+      </c>
+      <c r="H12" s="42">
+        <f>'Working Capital_Actual'!H4</f>
+        <v>36120.436180166136</v>
+      </c>
+      <c r="I12" s="42">
+        <f>'Working Capital_Actual'!I4</f>
+        <v>9803.0302230313246</v>
+      </c>
+      <c r="J12" s="42">
+        <f>'Working Capital_Actual'!J4</f>
+        <v>9235</v>
+      </c>
+      <c r="K12" s="42">
+        <f>'Working Capital_Actual'!K4</f>
+        <v>10863.810550512382</v>
+      </c>
+      <c r="L12" s="42">
+        <f>'Working Capital_Actual'!L4</f>
+        <v>12568</v>
+      </c>
+      <c r="M12" s="42">
+        <f>'Working Capital_Actual'!M4</f>
+        <v>11506</v>
+      </c>
+      <c r="N12" s="42">
+        <f>'Working Capital_Actual'!N4</f>
+        <v>14111</v>
+      </c>
+      <c r="O12" s="42">
+        <v>0</v>
+      </c>
+      <c r="P12" s="42">
+        <v>0</v>
+      </c>
+      <c r="Q12" s="42">
+        <v>0</v>
+      </c>
+      <c r="R12" s="42">
+        <v>0</v>
+      </c>
+      <c r="S12" s="42">
+        <v>0</v>
+      </c>
+      <c r="T12" s="42">
+        <v>0</v>
+      </c>
+      <c r="U12" s="42">
+        <v>0</v>
+      </c>
+      <c r="V12" s="42">
+        <v>0</v>
+      </c>
+      <c r="W12" s="42">
+        <v>0</v>
+      </c>
+      <c r="X12" s="42">
+        <v>0</v>
+      </c>
+      <c r="Y12" s="42">
+        <v>0</v>
+      </c>
+      <c r="Z12" s="42">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="A13" s="12" t="s">
+        <v>93</v>
+      </c>
+      <c r="B13" s="42">
+        <v>0</v>
+      </c>
+      <c r="C13" s="42">
+        <v>0</v>
+      </c>
+      <c r="D13" s="42">
+        <v>0</v>
+      </c>
+      <c r="E13" s="42">
+        <v>0</v>
+      </c>
+      <c r="F13" s="42">
+        <v>0</v>
+      </c>
+      <c r="G13" s="42">
+        <v>0</v>
+      </c>
+      <c r="H13" s="42">
+        <v>0</v>
+      </c>
+      <c r="I13" s="42">
+        <v>0</v>
+      </c>
+      <c r="J13" s="42">
+        <v>0</v>
+      </c>
+      <c r="K13" s="42">
+        <v>0</v>
+      </c>
+      <c r="L13" s="42">
+        <v>0</v>
+      </c>
+      <c r="M13" s="42">
+        <v>0</v>
+      </c>
+      <c r="N13" s="42">
+        <v>0</v>
+      </c>
+      <c r="O13" s="42">
+        <v>0</v>
+      </c>
+      <c r="P13" s="42">
+        <v>0</v>
+      </c>
+      <c r="Q13" s="42">
+        <v>0</v>
+      </c>
+      <c r="R13" s="42">
+        <v>0</v>
+      </c>
+      <c r="S13" s="42">
+        <v>0</v>
+      </c>
+      <c r="T13" s="42">
+        <v>0</v>
+      </c>
+      <c r="U13" s="42">
+        <v>0</v>
+      </c>
+      <c r="V13" s="42">
+        <v>0</v>
+      </c>
+      <c r="W13" s="42">
+        <v>0</v>
+      </c>
+      <c r="X13" s="42">
+        <v>0</v>
+      </c>
+      <c r="Y13" s="42">
+        <v>0</v>
+      </c>
+      <c r="Z13" s="42">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="A14" s="12" t="s">
+        <v>94</v>
+      </c>
+      <c r="B14" s="42">
+        <f>B10+B12+B13</f>
+        <v>54982.535294664027</v>
+      </c>
+      <c r="C14" s="42">
+        <f t="shared" ref="C14:N14" si="8">C10+C12+C13</f>
+        <v>33185.389800667006</v>
+      </c>
+      <c r="D14" s="42">
+        <f t="shared" si="8"/>
+        <v>49077.648605494804</v>
+      </c>
+      <c r="E14" s="42">
+        <f t="shared" si="8"/>
+        <v>6967.9673967445342</v>
+      </c>
+      <c r="F14" s="42">
+        <f t="shared" si="8"/>
+        <v>22990.427847235434</v>
+      </c>
+      <c r="G14" s="42">
+        <f t="shared" si="8"/>
+        <v>58687.193398158517</v>
+      </c>
+      <c r="H14" s="42">
+        <f t="shared" si="8"/>
+        <v>64120.436180166136</v>
+      </c>
+      <c r="I14" s="42">
+        <f t="shared" si="8"/>
+        <v>51803.030223031325</v>
+      </c>
+      <c r="J14" s="42">
+        <f t="shared" si="8"/>
+        <v>51235</v>
+      </c>
+      <c r="K14" s="42">
+        <f t="shared" si="8"/>
+        <v>42863.810550512382</v>
+      </c>
+      <c r="L14" s="42">
+        <f t="shared" si="8"/>
+        <v>12568</v>
+      </c>
+      <c r="M14" s="42">
+        <f t="shared" si="8"/>
+        <v>11506</v>
+      </c>
+      <c r="N14" s="42">
+        <f t="shared" si="8"/>
+        <v>14111</v>
+      </c>
+      <c r="O14" s="42">
+        <v>0</v>
+      </c>
+      <c r="P14" s="42">
+        <v>0</v>
+      </c>
+      <c r="Q14" s="42">
+        <v>0</v>
+      </c>
+      <c r="R14" s="42">
+        <v>0</v>
+      </c>
+      <c r="S14" s="42">
+        <v>0</v>
+      </c>
+      <c r="T14" s="42">
+        <v>0</v>
+      </c>
+      <c r="U14" s="42">
+        <v>0</v>
+      </c>
+      <c r="V14" s="42">
+        <v>0</v>
+      </c>
+      <c r="W14" s="42">
+        <v>0</v>
+      </c>
+      <c r="X14" s="42">
+        <v>0</v>
+      </c>
+      <c r="Y14" s="42">
+        <v>0</v>
+      </c>
+      <c r="Z14" s="42">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="A15" s="12" t="s">
+        <v>95</v>
+      </c>
+      <c r="B15" s="42">
+        <v>54982.535294664027</v>
+      </c>
+      <c r="C15" s="42">
+        <v>33185.389800667006</v>
+      </c>
+      <c r="D15" s="42">
+        <v>49077.648605494804</v>
+      </c>
+      <c r="E15" s="42">
+        <v>6967.9673967445342</v>
+      </c>
+      <c r="F15" s="42">
+        <v>22990.427847235434</v>
+      </c>
+      <c r="G15" s="42">
+        <v>58687.193398158517</v>
+      </c>
+      <c r="H15" s="42">
+        <v>64120.436180166136</v>
+      </c>
+      <c r="I15" s="42">
+        <v>51803.030223031325</v>
+      </c>
+      <c r="J15" s="42">
+        <v>51235</v>
+      </c>
+      <c r="K15" s="42">
+        <v>42863.810550512382</v>
+      </c>
+      <c r="L15" s="42">
+        <v>12568</v>
+      </c>
+      <c r="M15" s="42">
+        <v>11506</v>
+      </c>
+      <c r="N15" s="42">
+        <v>14111</v>
+      </c>
+      <c r="O15" s="42">
+        <v>0</v>
+      </c>
+      <c r="P15" s="42">
+        <v>0</v>
+      </c>
+      <c r="Q15" s="42">
+        <v>0</v>
+      </c>
+      <c r="R15" s="42">
+        <v>0</v>
+      </c>
+      <c r="S15" s="42">
+        <v>0</v>
+      </c>
+      <c r="T15" s="42">
+        <v>0</v>
+      </c>
+      <c r="U15" s="42">
+        <v>0</v>
+      </c>
+      <c r="V15" s="42">
+        <v>0</v>
+      </c>
+      <c r="W15" s="42">
+        <v>0</v>
+      </c>
+      <c r="X15" s="42">
+        <v>0</v>
+      </c>
+      <c r="Y15" s="42">
+        <v>0</v>
+      </c>
+      <c r="Z15" s="42">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="A16" s="12" t="s">
+        <v>96</v>
+      </c>
+      <c r="B16" s="42">
+        <v>355000</v>
+      </c>
+      <c r="C16" s="42">
+        <v>355000</v>
+      </c>
+      <c r="D16" s="42">
+        <v>355000</v>
+      </c>
+      <c r="E16" s="42">
+        <v>355000</v>
+      </c>
+      <c r="F16" s="42">
+        <v>355000</v>
+      </c>
+      <c r="G16" s="42">
+        <v>355000</v>
+      </c>
+      <c r="H16" s="42">
+        <v>355000</v>
+      </c>
+      <c r="I16" s="42">
+        <v>355000</v>
+      </c>
+      <c r="J16" s="42">
+        <v>355000</v>
+      </c>
+      <c r="K16" s="42">
+        <v>355000</v>
+      </c>
+      <c r="L16" s="42">
+        <v>355000</v>
+      </c>
+      <c r="M16" s="42">
+        <v>355000</v>
+      </c>
+      <c r="N16" s="42">
+        <v>355000</v>
+      </c>
+      <c r="O16" s="42">
+        <v>0</v>
+      </c>
+      <c r="P16" s="42">
+        <v>0</v>
+      </c>
+      <c r="Q16" s="42">
+        <v>0</v>
+      </c>
+      <c r="R16" s="42">
+        <v>0</v>
+      </c>
+      <c r="S16" s="42">
+        <v>0</v>
+      </c>
+      <c r="T16" s="42">
+        <v>0</v>
+      </c>
+      <c r="U16" s="42">
+        <v>0</v>
+      </c>
+      <c r="V16" s="42">
+        <v>0</v>
+      </c>
+      <c r="W16" s="42">
+        <v>0</v>
+      </c>
+      <c r="X16" s="42">
+        <v>0</v>
+      </c>
+      <c r="Y16" s="42">
+        <v>0</v>
+      </c>
+      <c r="Z16" s="42">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.26" right="0.70866141732283472" top="0.28999999999999998" bottom="0.2" header="0.2" footer="0.31496062992125984"/>
+  <pageSetup paperSize="9" orientation="landscape" verticalDpi="0" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -8939,7 +11596,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:Z36"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="15.05" x14ac:dyDescent="0.3"/>
@@ -12572,7 +15229,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:LH4"/>
   <sheetFormatPr defaultRowHeight="15.05" x14ac:dyDescent="0.3"/>
@@ -12913,7 +15570,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -14526,7 +17183,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:Z20"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="11.3" x14ac:dyDescent="0.2"/>
@@ -16361,7 +19018,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -17412,7 +20069,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:AA17"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="11.3" x14ac:dyDescent="0.2"/>

</xml_diff>